<commit_message>
Wire lists: ends with no cavity say Splice / Terminal / Screen instead of a blank pin
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1085,7 +1085,11 @@
           <t>SP-CAM</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>Cam sensor signal</t>
@@ -2265,7 +2269,11 @@
           <t>SP-GND-ECU</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>ECU power ground</t>
@@ -2855,7 +2863,11 @@
           <t>SP-GND-ECU</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>ECU power ground</t>
@@ -3231,7 +3243,11 @@
           <t>SP-TACH</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Engine speed (tacho)</t>
@@ -4092,7 +4108,11 @@
           <t>SP-AC-SG</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>Ambient sensor return</t>
@@ -4294,7 +4314,11 @@
           <t>POWER-NEG-BAR</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>A/C coolant-OK ground</t>
@@ -4496,7 +4520,11 @@
           <t>SP-AC-PSW</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>A/C pressure sw out</t>
@@ -4601,7 +4629,11 @@
           <t>SP-AC-PSW</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>A/C pressure sw out</t>
@@ -6895,7 +6927,11 @@
           <t>SP-SW12</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse</t>
@@ -6988,7 +7024,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>screen</t>
+          <t>Screen</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6996,7 +7032,11 @@
           <t>SP-SHIELD-A-APS</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>Pedal 1 cable shield</t>
@@ -7089,7 +7129,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>screen</t>
+          <t>Screen</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7097,7 +7137,11 @@
           <t>SP-SHIELD-A-APS</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>Pedal 2 cable shield</t>
@@ -7190,7 +7234,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>screen</t>
+          <t>Screen</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7198,7 +7242,11 @@
           <t>SP-SHIELD-A-WSF</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>FR wheel spd shield</t>
@@ -7299,7 +7347,11 @@
           <t>SP-A5</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse (+ IG2 wake diode)</t>
@@ -7396,7 +7448,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
           <t>Flex fuel shield</t>
@@ -7493,7 +7549,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>Throttle shield</t>
@@ -7590,7 +7650,11 @@
           <t>SP-SHIELD-B</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>ETB motor shield</t>
@@ -7683,7 +7747,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>Turbo speed shield</t>
@@ -7780,7 +7848,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>Cam sensor shield</t>
@@ -7970,7 +8042,11 @@
           <t>SP-SHIELD-B</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr">
         <is>
           <t>Gearbox speed shield</t>
@@ -8164,7 +8240,11 @@
           <t>SP-SHIELD-B</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>Knock sensor shield</t>
@@ -8257,7 +8337,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>Crank sensor shield</t>
@@ -8358,7 +8442,11 @@
           <t>SP-REV</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>Reverse sw +12 V out</t>
@@ -8455,7 +8543,11 @@
           <t>POWER-NEG-BAR</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>CAN-Lambda ground</t>
@@ -8653,7 +8745,11 @@
           <t>SP-FUEL-LVL</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>Fuel level signal</t>
@@ -9283,7 +9379,11 @@
           <t>SP-SHIELD-A-WSF</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>WS-F screen drain</t>
@@ -9804,7 +9904,11 @@
           <t>SP-SHIELD-B-WSR</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>WS-R screen drain</t>
@@ -11281,13 +11385,21 @@
           <t>POWER-NEG-BAR</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>SP-CSB-GND</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
           <t>CSB3 + opto ground</t>
@@ -11388,7 +11500,11 @@
           <t>SP-CAM</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>Cam pull-up 1.8k</t>
@@ -11766,7 +11882,11 @@
           <t>SP-8V</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D114" t="inlineStr">
         <is>
           <t>ECU-A</t>
@@ -11863,7 +11983,11 @@
           <t>SP-8V</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D115" t="inlineStr">
         <is>
           <t>R-CAM-PULLUP</t>
@@ -11956,7 +12080,11 @@
           <t>SP-8V</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D116" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -12053,7 +12181,11 @@
           <t>SP-A5</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D117" t="inlineStr">
         <is>
           <t>ECU-A</t>
@@ -12154,7 +12286,11 @@
           <t>SP-AC-SG</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D118" t="inlineStr">
         <is>
           <t>A32</t>
@@ -12255,7 +12391,11 @@
           <t>SP-ACC12</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D119" t="inlineStr">
         <is>
           <t>K-ACC</t>
@@ -12356,7 +12496,11 @@
           <t>SP-CAM</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D120" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -12453,7 +12597,11 @@
           <t>SP-CAN-SH-BH</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D121" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -12554,7 +12702,11 @@
           <t>SP-CANH</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D122" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -12659,7 +12811,11 @@
           <t>SP-CANL</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D123" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -12764,7 +12920,11 @@
           <t>SP-FUEL-LVL</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D124" t="inlineStr">
         <is>
           <t>R-FUELLVL</t>
@@ -12853,7 +13013,11 @@
           <t>SP-FUEL-LVL</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D125" t="inlineStr">
         <is>
           <t>ECU-B</t>
@@ -12946,13 +13110,21 @@
           <t>SP-GND-ECU</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>POWER-NEG-BAR</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
       <c r="F126" t="inlineStr">
         <is>
           <t>ECU power ground</t>
@@ -13043,7 +13215,11 @@
           <t>SP-GND-ECU</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>ECU-B</t>
@@ -13144,7 +13320,11 @@
           <t>SP-GND-ECU</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D128" t="inlineStr">
         <is>
           <t>ECU-B</t>
@@ -13245,7 +13425,11 @@
           <t>SP-REV</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D129" t="inlineStr">
         <is>
           <t>IG2</t>
@@ -13346,7 +13530,11 @@
           <t>SP-REV</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D130" t="inlineStr">
         <is>
           <t>OPTO-8</t>
@@ -13443,7 +13631,11 @@
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D131" t="inlineStr">
         <is>
           <t>ECU-A</t>
@@ -13544,13 +13736,21 @@
           <t>SP-SHIELD-A-APS</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F132" t="inlineStr">
         <is>
           <t>Shield drain</t>
@@ -13637,13 +13837,21 @@
           <t>SP-SHIELD-A-WSF</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>SP-SHIELD-A</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F133" t="inlineStr">
         <is>
           <t>Shield drain</t>
@@ -13730,7 +13938,11 @@
           <t>SP-SHIELD-B</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>ECU-B</t>
@@ -13823,13 +14035,21 @@
           <t>SP-SHIELD-B-WSR</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
           <t>SP-SHIELD-B</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
           <t>Shield drain B</t>
@@ -13916,13 +14136,21 @@
           <t>SP-SW12</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D136" t="inlineStr">
         <is>
           <t>SP-A5</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="F136" t="inlineStr">
         <is>
           <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse (+ IG2 wake diode)</t>
@@ -14013,7 +14241,11 @@
           <t>SP-SW12</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D137" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -14114,7 +14346,11 @@
           <t>SP-SW12</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D138" t="inlineStr">
         <is>
           <t>DRB102-CABIN</t>
@@ -14215,7 +14451,11 @@
           <t>SP-TACH</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D139" t="inlineStr">
         <is>
           <t>A18</t>
@@ -14320,7 +14560,11 @@
           <t>SP-TACH</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Splice</t>
+        </is>
+      </c>
       <c r="D140" t="inlineStr">
         <is>
           <t>R-LOCK</t>
@@ -18608,7 +18852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -18652,12 +18896,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Contact PN 'solder splice' / 'solder onto the factory lead' = no contact; TBD = not confirmed by a maker document.</t>
+          <t>Pin 'Splice' / 'Terminal' / 'Screen' = an end with no cavity (a solder splice, a ring or spade lug, a cable screen).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>Contact PN 'solder splice' / 'solder onto the factory lead' = no contact; TBD = not confirmed by a maker document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Wires: 139   Connectors / ends: 59   Splices: 20   Spare cavities: 61</t>
         </is>

</xml_diff>

<commit_message>
Wire lists: read-back gate against the master; source / factory-tap trunk steps
--check now reads each committed wire list back (every wire once, device ends and pins, gauge,
colour, bands; no splice or blank in From / To; one trunk per splice). The digest covers the whole
master. DECISIONS "Wire lists" rule 4 and 8 updated. OPEN-ITEMS: audit results and the W1 washer
end found in EngineRoom-C.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -11827,12 +11827,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>K-ACC</t>
+          <t>LOGIC</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>BUS2-8</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -18914,7 +18914,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>w_fb_k_acc_30_cp</t>
+          <t>w_acc_fuse</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
ECU engine harness: crank / cam shielded cables, CAN-Lambda branch, starter bulkhead pin (Rev I)
- Crank: one 2-core shielded cable; cam: one 3-core (no loose wires in a shielded run).
- CAN-Lambda branch owned by AB-engine: shielded pair to the splices and 120R terminator behind the plug.
- Starter S on DRB102 cavity 3, 12 AWG, size-12 contacts (w_strl_c CabinPower / w_strl_e AB-engine).
- ECU-B 10 tach contact 3-1447221-4 (20 AWG); check_wiring M2 now reads single-size contact ranges.
- Drawings, wire lists, DRB map and BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Connectors'!$A$1:$I$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Splices'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16284,7 +16284,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -16730,7 +16730,7 @@
         <v>64</v>
       </c>
       <c r="H9" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -19248,7 +19248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19529,7 +19529,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -19551,7 +19551,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19573,7 +19573,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -19639,12 +19639,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0413-214-1205</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -19661,7 +19661,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -19683,7 +19683,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -19705,7 +19705,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -19727,7 +19727,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -19749,7 +19749,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -19771,7 +19771,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -19793,7 +19793,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -19815,12 +19815,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>114019-ZZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -19837,12 +19837,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>114019-ZZ</t>
+          <t>114018-ZZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -19859,7 +19859,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -19881,12 +19881,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>114018-ZZ</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -19903,12 +19903,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>114018-ZZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -19925,7 +19925,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -19947,12 +19947,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>114018-ZZ</t>
+          <t>114019-ZZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -19969,12 +19969,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>62</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>114019-ZZ</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -19991,7 +19991,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -20013,7 +20013,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>86</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -20035,7 +20035,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -20057,7 +20057,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -20101,7 +20101,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -20123,7 +20123,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -20189,7 +20189,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -20211,12 +20211,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>97</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>0413-214-1205</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -20233,7 +20233,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -20255,7 +20255,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -20277,7 +20277,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -20299,7 +20299,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>101</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -20321,7 +20321,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>102</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -20338,34 +20338,34 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DRB102-CABIN</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0413-214-1205</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
+          <t>spare, not used</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -20387,7 +20387,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -20409,7 +20409,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -20453,7 +20453,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -20475,7 +20475,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -20497,7 +20497,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -20519,7 +20519,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -20558,29 +20558,29 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>IX-WS-F-S</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>spare, not used</t>
+          <t>spare, sealing plug</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>IX-WS-F-S</t>
+          <t>IX-WS-R-S</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -20599,30 +20599,8 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>IX-WS-R-S</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>114017</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D62"/>
+  <autoFilter ref="A1:D61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20712,7 +20690,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wires: 139   Connectors / ends: 59   Splices: 20   Spare cavities: 61</t>
+          <t>Wires: 139   Connectors / ends: 59   Splices: 20   Spare cavities: 60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CAN-Lambda power / ground leads 20 -> 16 AWG in 0462-005-2031 sockets (row 168)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014aA8s5xrHBiGf55NfPQAJv
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$140</definedName>

</xml_diff>

<commit_message>
CAN-Lambda power / ground leads 20 -> 16 AWG in 0462-005-2031 sockets (row 168) (#418)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014aA8s5xrHBiGf55NfPQAJv
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$140</definedName>

</xml_diff>

<commit_message>
w_fp85: cabin run to the trunk relay block, est 2890 mm (row 157)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014aA8s5xrHBiGf55NfPQAJv
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -12651,7 +12651,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -12699,13 +12699,13 @@
       <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>glove-box branch (POWER / LOGIC boxes) / cabin run to the trunk relay block (Routes 1 / 11)</t>
         </is>
       </c>
       <c r="Y108" t="inlineStr"/>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85 | owner proposed: longer half (drawn today as w_fp85 on ECU-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
+          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85 | est length: ECU-A to the glove-box boxes (390 mm) plus the cabin run to K-FP in the trunk relay block, alongside w_k_fp_86_cp (2500 mm); row 157</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
w_fp85: cabin run to the trunk relay block, est 2890 mm (row 157) (#419)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014aA8s5xrHBiGf55NfPQAJv
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -12651,7 +12651,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -12699,13 +12699,13 @@
       <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>glove-box branch (POWER / LOGIC boxes) / cabin run to the trunk relay block (Routes 1 / 11)</t>
         </is>
       </c>
       <c r="Y108" t="inlineStr"/>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85 | owner proposed: longer half (drawn today as w_fp85 on ECU-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
+          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85 | est length: ECU-A to the glove-box boxes (390 mm) plus the cabin run to K-FP in the trunk relay block, alongside w_k_fp_86_cp (2500 mm); row 157</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EPS pump signal wires owned by the ECU engine harness (+203 mm bulkhead drop)
Dan 2026-10-29 (A10): w_hv_mrs_en_e, w_mrs_e and w_eps_rly_e leave engine bulkhead cavities 83-85 in the
engine loom, so AB-engine owns them (were EngineRoom-C passing through AB-engine); harness C keeps the
8 AWG pump power and ground. Their lengths pick up the 203 mm bulkhead drop (652 -> 855).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -2602,7 +2602,7 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>ST185-EngineRoom-C w_mrs_e at DRB102-ENGINE 84, to MRS-B 2</t>
+          <t>ST185-AB-engine w_mrs_e at DRB102-ENGINE 84, to MRS-B 2</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -12258,7 +12258,7 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>ST185-EngineRoom-C w_eps_rly_e at DRB102-ENGINE 85, to MRS-B 5</t>
+          <t>ST185-AB-engine w_eps_rly_e at DRB102-ENGINE 85, to MRS-B 5</t>
         </is>
       </c>
       <c r="X104" t="inlineStr">
@@ -13038,7 +13038,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>ST185-EngineRoom-C w_hv_mrs_en_e at DRB102-ENGINE 83, to MRS-C 1</t>
+          <t>ST185-AB-engine w_hv_mrs_en_e at DRB102-ENGINE 83, to MRS-C 1</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">

</xml_diff>

<commit_message>
CAN cables: Raychem 55A1821-20-9/5-9 (was TBD)
Dan 2026-10-29 (A9): every CAN cable is a two-core shielded Raychem cable at a gauge fit for the load.
55A1821-20 is a 20 AWG twisted pair with a tinned-copper braid and ETFE jacket (TE); white / green cores
match CAN H / CAN L; 20 AWG suits the size-20 contacts (CAN draws milliamps). 18 rows; parts table +1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -9706,7 +9706,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-20-9/5-9</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -9830,7 +9830,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-20-9/5-9</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
@@ -9950,7 +9950,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-20-9/5-9</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">

</xml_diff>

<commit_message>
Coolant pressure pins A/B/C, cam sensor GS1007 note, Needs Dan N65-N68
- Master + device reference: coolant pressure pins 1/2/3 -> A/B/C (Dan's sensor sheet: A GND, B supply, C output; Dan OK).
- Cam rows: Cherry (ZF) GS1007 hall from the Racer X kit, leads brown +V / black signal / blue ground.
- OPEN-ITEMS: Current state, rows 130 / 150, History; Needs Dan N65 (ETB contacts 24-20 AWG vs 18 AWG motor pair),
  N66 (coolant pigtail), N67 (starter S plug), N68 (cam lead gauge).
- Drawing set, wire lists and BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -4130,7 +4130,7 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>ST185-AB-engine w35_e at DRB102-ENGINE 26, to CLNT-P 3</t>
+          <t>ST185-AB-engine w35_e at DRB102-ENGINE 26, to CLNT-P C</t>
         </is>
       </c>
       <c r="X33" t="inlineStr"/>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>ST185-AB-engine w_5v_brail_e_c47 at DRB102-ENGINE 25, to CLNT-P 2</t>
+          <t>ST185-AB-engine w_5v_brail_e_c47 at DRB102-ENGINE 25, to CLNT-P B</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">

</xml_diff>

<commit_message>
ETB motor pair 18 -> 20 AWG on the Bosch kit contacts (Needs Dan N65)
Bosch ETB max generator current < 10 A; Link Aux 9/10 H-bridge 4 A;
kit contact MQS 0.63 (0.22-0.5 mm2), TE typical 7.5 A. ECU-B B18/B26 now
Superseal 3-1447221-4 (20 AWG), bulkhead size-16 contacts unchanged,
engine side 55A1821-20-2/0-9. ETB pins cite the Bosch pin table.
Drawing set, wirelists and BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$141</definedName>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3876,14 +3876,14 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4312,14 +4312,14 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">

</xml_diff>

<commit_message>
ETB motor pair 18 -> 20 AWG on the Bosch kit contacts (Needs Dan N65) (#422)
Bosch ETB max generator current < 10 A; Link Aux 9/10 H-bridge 4 A;
kit contact MQS 0.63 (0.22-0.5 mm2), TE typical 7.5 A. ECU-B B18/B26 now
Superseal 3-1447221-4 (20 AWG), bulkhead size-16 contacts unchanged,
engine side 55A1821-20-2/0-9. ETB pins cite the Bosch pin table.
Drawing set, wirelists and BOM regenerated.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$141</definedName>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3876,14 +3876,14 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4312,14 +4312,14 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">

</xml_diff>

<commit_message>
Coolant pressure pigtail in the master (N66), starter / reverse plug notes (N67)
- CLNT-P: pigtail supplied with the sensor; plug 1 GND black / 2 supply red / 3 output green = A / B / C;
  harness solder-splices to the leads (Dan's seller-guide photos). Row 130 closed.
- Starter S: candidate 90980-11400 (Toyota RM1022E: 1-way sealed, 4.8 mm tab); N67 asks for a tab check.
- Reverse switch: 90980-11250 confirmed 2.3 II mm female 2-way sealed (RM1022E); kit owned.
- Device reference, OPEN-ITEMS (Current state, rows 130 / 140, Needs Dan, History); drawings, wire lists, BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$141</definedName>

</xml_diff>

<commit_message>
ETB motor pair 20 -> 16 AWG (Bosch 10 A limit), short 20 AWG tails at the ETB plug
- Bosch ETB data sheet: motor current up to 10 A. M22759/16 at 100 C ambient: 20 AWG 6 A, 18 AWG 9 A, 16 AWG 12 A
  (HP Academy cheat sheet), so 20 AWG (#422) was too small.
- Cabin w124_c / w215_c: M22759/16-16-9 in ECU contact 3-1447221-3 (TE: 0.75-1.25 mm2, 18-16 AWG, insul 1.6-2.2 mm).
- Bulkhead size-16 contacts take 16-20 AWG (no change).
- Engine pair: 55A1821-16-2/0-9; cores splice to short 20 AWG tails at the ETB plug (kit contact 24-20 AWG only).
- Parts table: cable renamed, 16 AWG white added, Superseal 3-1447221-3 text corrected. OPEN-ITEMS History / state.
- Drawings, wire lists, BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -3866,7 +3866,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3876,14 +3876,14 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>M22759/16-16-9</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>3-1447221-3</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4312,14 +4312,14 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>M22759/16-16-9</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>3-1447221-3</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">

</xml_diff>

<commit_message>
LOGIC SW12 and MRS fuses 7.5 -> 5 A for the 20 AWG engine-bay wires (wire vs fuse audit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -7715,7 +7715,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse (+ IG2 wake diode)</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -8059,7 +8059,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -12971,7 +12971,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC MRS 7.5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC MRS 5 A fuse</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse (+ IG2 wake diode)</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -16247,7 +16247,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 7.5 A fuse (+ IG2 wake diode)</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">

</xml_diff>

<commit_message>
Wire/fuse audit applied (Dan N72-N77, B12): coils, injectors, horns, ETB, fuel pump ground
- Coils: 14 AWG trunk both sides, 16 AWG power and ground branches, COP fuse 15 -> 10 A
- Injectors: 14 AWG engine trunk, INJ fuse 15 -> 7.5 A
- Horns (PIAA Slim): 14 AWG whole run, DT 14 AWG sockets 0462-209-16141, D-436-38 splice
- ETB motor: 18 AWG whole circuit, TE 5-965906-1 at the ETB (test-fit pending), ETB fuse 7.5 A
- Fuel pump ground 12 -> 10 AWG; pump's own lead noted
- DECISIONS B12 cases; OPEN-ITEMS N78 fans, N79 FP fuse; drawings, BOM, fuse-box plan regenerated/synced

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -3866,7 +3866,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-16-9</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-16-9</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -8017,7 +8017,7 @@
       <c r="Y67" t="inlineStr"/>
       <c r="Z67" t="inlineStr">
         <is>
-          <t>(firewall bulkhead, RH) | M8 ring lug on the POWER box battery-negative bar (Dan 2026-10-29: coil ground, cleanest return) | est length; runs with the coil +12 V (w_cop_pwr_ac, LOGIC COP 15 A) from the glove box to bulkhead pin 1 / 4; 14 AWG like that feed</t>
+          <t>(firewall bulkhead, RH) | M8 ring lug on the POWER box battery-negative bar (Dan 2026-10-29: coil ground, cleanest return) | est length; runs with the coil +12 V (w_cop_pwr_ac, LOGIC COP 10 A) from the glove box to bulkhead pin 1 / 4; 14 AWG like that feed</t>
         </is>
       </c>
     </row>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC COP 15 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC COP 10 A fuse</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -13273,7 +13273,7 @@
       <c r="Y113" t="inlineStr"/>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse COP 15A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse COP 10A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm)</t>
         </is>
       </c>
     </row>
@@ -13311,7 +13311,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC INJ 15 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC INJ 7.5 A fuse</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -13389,7 +13389,7 @@
       <c r="Y114" t="inlineStr"/>
       <c r="Z114" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse INJ 15A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse INJ 7.5A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire type: SAE J1128 TXL in cabin, trunk and harness-C low-current runs (Dan N82 A, B20)
- 196 master rows M22759/16 -> J1128-TXL-<awg>-<colour>; Tefzel stays on AB-engine, near exhaust/turbo,
  Spec 55 cables, and 20 circuits where derated TXL (0.8x cabin, 0.7x engine bay) is below the fuse
- DECISIONS B20; harness-parts TXL rows; tracker N82 closed, N81 updated; drawings and BOM regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -880,7 +880,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -992,7 +992,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>M22759/16-18-6</t>
+          <t>J1128-TXL-18-BLUE</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N21" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>M22759/16-18-3</t>
+          <t>J1128-TXL-18-ORANGE</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>M22759/16-18-6</t>
+          <t>J1128-TXL-18-BLUE</t>
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N38" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N39" t="inlineStr"/>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="N40" t="inlineStr"/>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N61" t="inlineStr"/>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N62" t="inlineStr"/>
@@ -7512,7 +7512,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N63" t="inlineStr"/>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N64" t="inlineStr"/>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N65" t="inlineStr"/>
@@ -7856,7 +7856,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N66" t="inlineStr"/>
@@ -7964,7 +7964,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>J1128-TXL-14-BLACK</t>
         </is>
       </c>
       <c r="N67" t="inlineStr"/>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N68" t="inlineStr"/>
@@ -8664,7 +8664,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N73" t="inlineStr"/>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N74" t="inlineStr"/>
@@ -9012,7 +9012,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>J1128-TXL-14-BLACK</t>
         </is>
       </c>
       <c r="N85" t="inlineStr"/>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>J1128-TXL-16-RED</t>
         </is>
       </c>
       <c r="N86" t="inlineStr"/>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N87" t="inlineStr"/>
@@ -10416,7 +10416,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N88" t="inlineStr"/>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N89" t="inlineStr"/>
@@ -11768,7 +11768,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N100" t="inlineStr"/>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N101" t="inlineStr"/>
@@ -12104,7 +12104,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N103" t="inlineStr"/>
@@ -12444,7 +12444,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N106" t="inlineStr"/>
@@ -12884,7 +12884,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N110" t="inlineStr"/>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N111" t="inlineStr"/>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N112" t="inlineStr"/>
@@ -13220,7 +13220,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N113" t="inlineStr"/>
@@ -13336,7 +13336,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N114" t="inlineStr"/>
@@ -13456,7 +13456,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N115" t="inlineStr"/>
@@ -13572,7 +13572,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N116" t="inlineStr"/>
@@ -13680,7 +13680,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N117" t="inlineStr"/>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N118" t="inlineStr"/>
@@ -13888,7 +13888,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N119" t="inlineStr"/>
@@ -13992,7 +13992,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N120" t="inlineStr"/>
@@ -14100,7 +14100,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N121" t="inlineStr"/>
@@ -14212,7 +14212,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N122" t="inlineStr"/>
@@ -14676,7 +14676,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N126" t="inlineStr"/>
@@ -14788,7 +14788,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N127" t="inlineStr"/>
@@ -15024,7 +15024,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N129" t="inlineStr"/>
@@ -15140,7 +15140,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N130" t="inlineStr"/>
@@ -15252,7 +15252,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="N131" t="inlineStr"/>
@@ -15372,7 +15372,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N132" t="inlineStr"/>
@@ -15480,7 +15480,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>M22759/16-10-0</t>
+          <t>J1128-TXL-10-BLACK</t>
         </is>
       </c>
       <c r="N133" t="inlineStr"/>
@@ -15596,7 +15596,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N134" t="inlineStr"/>
@@ -16272,7 +16272,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N140" t="inlineStr"/>
@@ -16388,7 +16388,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N141" t="inlineStr"/>

</xml_diff>

<commit_message>
Wire type: SAE J1128 TXL in cabin, trunk and harness-C low-current runs (Dan N82 A, B20) (#429)
- 196 master rows M22759/16 -> J1128-TXL-<awg>-<colour>; Tefzel stays on AB-engine, near exhaust/turbo,
  Spec 55 cables, and 20 circuits where derated TXL (0.8x cabin, 0.7x engine bay) is below the fuse
- DECISIONS B20; harness-parts TXL rows; tracker N82 closed, N81 updated; drawings and BOM regenerated


Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -880,7 +880,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -992,7 +992,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>M22759/16-18-6</t>
+          <t>J1128-TXL-18-BLUE</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N21" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>M22759/16-18-3</t>
+          <t>J1128-TXL-18-ORANGE</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>M22759/16-18-6</t>
+          <t>J1128-TXL-18-BLUE</t>
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>J1128-TXL-18-BLACK</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N38" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N39" t="inlineStr"/>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="N40" t="inlineStr"/>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N61" t="inlineStr"/>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N62" t="inlineStr"/>
@@ -7512,7 +7512,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N63" t="inlineStr"/>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N64" t="inlineStr"/>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N65" t="inlineStr"/>
@@ -7856,7 +7856,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N66" t="inlineStr"/>
@@ -7964,7 +7964,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>J1128-TXL-14-BLACK</t>
         </is>
       </c>
       <c r="N67" t="inlineStr"/>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N68" t="inlineStr"/>
@@ -8664,7 +8664,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N73" t="inlineStr"/>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N74" t="inlineStr"/>
@@ -9012,7 +9012,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>J1128-TXL-14-BLACK</t>
         </is>
       </c>
       <c r="N85" t="inlineStr"/>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>J1128-TXL-16-RED</t>
         </is>
       </c>
       <c r="N86" t="inlineStr"/>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N87" t="inlineStr"/>
@@ -10416,7 +10416,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N88" t="inlineStr"/>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>J1128-TXL-20-BLUE</t>
         </is>
       </c>
       <c r="N89" t="inlineStr"/>
@@ -11768,7 +11768,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N100" t="inlineStr"/>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N101" t="inlineStr"/>
@@ -12104,7 +12104,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>J1128-TXL-18-WHITE</t>
         </is>
       </c>
       <c r="N103" t="inlineStr"/>
@@ -12444,7 +12444,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N106" t="inlineStr"/>
@@ -12884,7 +12884,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N110" t="inlineStr"/>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>M22759/16-20-2</t>
+          <t>J1128-TXL-20-RED</t>
         </is>
       </c>
       <c r="N111" t="inlineStr"/>
@@ -13112,7 +13112,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N112" t="inlineStr"/>
@@ -13220,7 +13220,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N113" t="inlineStr"/>
@@ -13336,7 +13336,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>M22759/16-14-2</t>
+          <t>J1128-TXL-14-RED</t>
         </is>
       </c>
       <c r="N114" t="inlineStr"/>
@@ -13456,7 +13456,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N115" t="inlineStr"/>
@@ -13572,7 +13572,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N116" t="inlineStr"/>
@@ -13680,7 +13680,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N117" t="inlineStr"/>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N118" t="inlineStr"/>
@@ -13888,7 +13888,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N119" t="inlineStr"/>
@@ -13992,7 +13992,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N120" t="inlineStr"/>
@@ -14100,7 +14100,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N121" t="inlineStr"/>
@@ -14212,7 +14212,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N122" t="inlineStr"/>
@@ -14676,7 +14676,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="N126" t="inlineStr"/>
@@ -14788,7 +14788,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N127" t="inlineStr"/>
@@ -15024,7 +15024,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="N129" t="inlineStr"/>
@@ -15140,7 +15140,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N130" t="inlineStr"/>
@@ -15252,7 +15252,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="N131" t="inlineStr"/>
@@ -15372,7 +15372,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N132" t="inlineStr"/>
@@ -15480,7 +15480,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>M22759/16-10-0</t>
+          <t>J1128-TXL-10-BLACK</t>
         </is>
       </c>
       <c r="N133" t="inlineStr"/>
@@ -15596,7 +15596,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="N134" t="inlineStr"/>
@@ -16272,7 +16272,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>M22759/16-18-2</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="N140" t="inlineStr"/>
@@ -16388,7 +16388,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="N141" t="inlineStr"/>

</xml_diff>

<commit_message>
Cleanup: fold CAN audit + setup checklist into CAN-BUS-MASTER-DESIGN, move 5sgte data, delete stale A/C page, trim tracker (Dan 2026-10-31)
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$141</definedName>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour G-Y; EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html); solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour G-Y; EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html); solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+          <t>EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cleanup: fold CAN audit + setup checklist into CAN-BUS-MASTER-DESIGN, move 5sgte data, delete stale A/C page, trim tracker (Dan 2026-10-31) (#437)
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$141</definedName>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour G-Y; EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html); solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour G-Y; EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html); solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+          <t>EWD 1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AB-cabin lengths from the layout tree, schematic banner page number fixed, rows 165/177 updated (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>820</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -4402,7 +4402,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>w_amb_rtn</t>
+          <t>w_amb_sig</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4422,22 +4422,18 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>SP-AC-SG</t>
-        </is>
-      </c>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>wire</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Ambient sensor return</t>
+          <t>Ambient temp signal</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4452,7 +4448,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -4469,17 +4465,17 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>solder splice SP-AC-SG</t>
+          <t>solder onto the factory lead</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
+          <t>OEM ambient air temp sensor A1 pin 2 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>via SP-AC-SG</t>
+          <t>OEM auto A/C amplifier A32 pin 6 TAM</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4494,31 +4490,31 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>Ambient air temp sensor A1 pin 2 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211 / p.148-150; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+          <t>B9 front pigtail. TAM signal to the auto A/C amp. Factory EA1/IQ1 path is gone.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>w_amb_sig</t>
+          <t>w_ac_cool_gnd</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4528,12 +4524,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A32</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -4544,12 +4540,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Ambient temp signal</t>
+          <t>A/C coolant-OK ground</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4559,39 +4555,39 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>860</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-YELLOW</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
+          <t>solder onto the factory lead</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t>320575</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 2 (front, 6 in pigtail)</t>
+          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>OEM auto A/C amplifier A32 pin 6 TAM</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACCGND</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -4601,26 +4597,30 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACCGND</t>
         </is>
       </c>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 2 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211 / p.148-150; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>A/C amplifier A18 (1993: A15) pin 2, behind the glove box; OEM colour L-Y; EWD 1993 p.210; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>B9 front pigtail. TAM signal to the auto A/C amp. Factory EA1/IQ1 path is gone.</t>
+          <t>D16: amp coolant-OK input hard-grounded. No Link ECT handshake.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>w_ac_cool_gnd</t>
+          <t>w_acc_trig</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4630,17 +4630,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>K-ACC</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -4651,27 +4651,27 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>A/C coolant-OK ground</t>
+          <t>A/C clutch relay coil (-)</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>860</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLACK</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>320575</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>B2-M5 A/C clutch relay (k_acc) - amp A15 pin 8 sinks coil- (85); coil+ (86) fused +12 V from B2-BUS2-8</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>ACCGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4708,30 +4708,26 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>ACCGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
+      <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15) pin 2, behind the glove box; OEM colour L-Y; EWD 1993 p.210; solder onto the factory lead</t>
+          <t>A/C amplifier A18 (1993: A15), behind the glove box; OEM colour L-Y; EWD 1993 p.210-211; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>D16: amp coolant-OK input hard-grounded. No Link ECT handshake.</t>
+          <t>A15 pin 8 MGC output (D16 option A). Solder onto the factory L-Y lead. | D16: amp drives k_acc coil 85. Link only sends ACT kill on Aux 4.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>w_acc_trig</t>
+          <t>w_ac_psw_sw</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4741,48 +4737,52 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>K-ACC</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SP-AC-PSW</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>leg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A/C clutch relay coil (-)</t>
+          <t>A/C pressure sw out</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4794,17 +4794,17 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>280919-2</t>
+          <t>solder splice SP-AC-PSW</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
+          <t>OEM A/C amplifier</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>B2-M5 A/C clutch relay (k_acc) - amp A15 pin 8 sinks coil- (85); coil+ (86) fused +12 V from B2-BUS2-8</t>
+          <t>via SP-AC-PSW</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4819,26 +4819,30 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15), behind the glove box; OEM colour L-Y; EWD 1993 p.210-211; solder onto the factory lead</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>A15 pin 8 MGC output (D16 option A). Solder onto the factory L-Y lead. | D16: amp drives k_acc coil 85. Link only sends ACT kill on Aux 4.</t>
+          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>w_ac_psw_sw</t>
+          <t>w_tach_18</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4848,22 +4852,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-TACH</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4873,12 +4877,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>Engine speed (tacho)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4888,12 +4892,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4905,22 +4909,22 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>solder splice SP-AC-PSW</t>
+          <t>solder splice SP-TACH</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier</t>
+          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>via SP-AC-PSW</t>
+          <t>via SP-TACH</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>TACH</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -4930,7 +4934,7 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-TACH</t>
         </is>
       </c>
       <c r="V42" t="inlineStr"/>
@@ -4941,44 +4945,44 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993: A15) pin 18, behind the glove box; OEM colour B; EWD 1993 p.211; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
+          <t>A15 pin 18 RPM input; 10-14 V average with the engine running (Mitchell 1993 Electrical). | D16: Ign 8 tacho to A15 pin 18.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>w_tach_18</t>
+          <t>w_amb_sg</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>A18</t>
+          <t>A32</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4988,12 +4992,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Engine speed (tacho)</t>
+          <t>A/C sensor common</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -5003,12 +5007,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
@@ -5020,22 +5024,22 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>solder splice SP-TACH</t>
+          <t>solder splice SP-AC-SG</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
+          <t>OEM auto A/C amplifier A32 pin 15 SG</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>via SP-TACH</t>
+          <t>via SP-AC-SG</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>TACH</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
@@ -5045,23 +5049,19 @@
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
+      <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15) pin 18, behind the glove box; OEM colour B; EWD 1993 p.211; solder onto the factory lead</t>
+          <t>Auto A/C amplifier A32 pin 15 SG, behind the glove box; OEM colour V-W; EWD 1993 p.211-212; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>A15 pin 18 RPM input; 10-14 V average with the engine running (Mitchell 1993 Electrical). | D16: Ign 8 tacho to A15 pin 18.</t>
+          <t>Cabin landing of SP-AC-SG on the amp sensor common.</t>
         </is>
       </c>
     </row>
@@ -5114,7 +5114,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>990</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -7409,7 +7409,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -9514,7 +9514,7 @@
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -9629,7 +9629,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -9740,7 +9740,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -9855,7 +9855,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -9970,7 +9970,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2820</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2820</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -10279,7 +10279,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>530</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>530</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -10616,7 +10616,7 @@
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -10834,7 +10834,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -11155,7 +11155,7 @@
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -12118,7 +12118,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -12221,7 +12221,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>3130</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -12875,7 +12875,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -12986,7 +12986,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -13089,7 +13089,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -13192,7 +13192,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -13703,7 +13703,7 @@
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -13814,7 +13814,7 @@
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -13925,7 +13925,7 @@
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -14258,7 +14258,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -14323,7 +14323,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>w_amb_sg</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -14338,12 +14338,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>A32</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>A/C sensor common</t>
+          <t>Ambient sensor return</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -14390,7 +14390,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -14400,7 +14400,7 @@
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>OEM auto A/C amplifier A32 pin 15 SG</t>
+          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
@@ -14422,12 +14422,12 @@
       <c r="W129" t="inlineStr"/>
       <c r="X129" t="inlineStr">
         <is>
-          <t>Auto A/C amplifier A32 pin 15 SG, behind the glove box; OEM colour V-W; EWD 1993 p.211-212; solder onto the factory lead</t>
+          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>Cabin landing of SP-AC-SG on the amp sensor common.</t>
+          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14484,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -14706,7 +14706,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -14809,7 +14809,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -15566,7 +15566,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -15677,7 +15677,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>820</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -18621,7 +18621,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>w_amb_sg</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">

</xml_diff>

<commit_message>
AB-cabin lengths from the layout tree, schematic banner page number fixed, rows 165/177 updated (Dan 2026-11-01) (#444)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>820</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -4402,7 +4402,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>w_amb_rtn</t>
+          <t>w_amb_sig</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4422,22 +4422,18 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>SP-AC-SG</t>
-        </is>
-      </c>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>wire</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Ambient sensor return</t>
+          <t>Ambient temp signal</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4452,7 +4448,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -4469,17 +4465,17 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>solder splice SP-AC-SG</t>
+          <t>solder onto the factory lead</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
+          <t>OEM ambient air temp sensor A1 pin 2 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>via SP-AC-SG</t>
+          <t>OEM auto A/C amplifier A32 pin 6 TAM</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4494,31 +4490,31 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>Ambient air temp sensor A1 pin 2 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211 / p.148-150; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+          <t>B9 front pigtail. TAM signal to the auto A/C amp. Factory EA1/IQ1 path is gone.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>w_amb_sig</t>
+          <t>w_ac_cool_gnd</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4528,12 +4524,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A32</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -4544,12 +4540,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Ambient temp signal</t>
+          <t>A/C coolant-OK ground</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4559,39 +4555,39 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>860</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-YELLOW</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
+          <t>solder onto the factory lead</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t>320575</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 2 (front, 6 in pigtail)</t>
+          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>OEM auto A/C amplifier A32 pin 6 TAM</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACCGND</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -4601,26 +4597,30 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACCGND</t>
         </is>
       </c>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 2 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211 / p.148-150; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>A/C amplifier A18 (1993: A15) pin 2, behind the glove box; OEM colour L-Y; EWD 1993 p.210; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>B9 front pigtail. TAM signal to the auto A/C amp. Factory EA1/IQ1 path is gone.</t>
+          <t>D16: amp coolant-OK input hard-grounded. No Link ECT handshake.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>w_ac_cool_gnd</t>
+          <t>w_acc_trig</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4630,17 +4630,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>K-ACC</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -4651,27 +4651,27 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>A/C coolant-OK ground</t>
+          <t>A/C clutch relay coil (-)</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>860</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLACK</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>320575</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>B2-M5 A/C clutch relay (k_acc) - amp A15 pin 8 sinks coil- (85); coil+ (86) fused +12 V from B2-BUS2-8</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>ACCGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4708,30 +4708,26 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>ACCGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
+      <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15) pin 2, behind the glove box; OEM colour L-Y; EWD 1993 p.210; solder onto the factory lead</t>
+          <t>A/C amplifier A18 (1993: A15), behind the glove box; OEM colour L-Y; EWD 1993 p.210-211; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>D16: amp coolant-OK input hard-grounded. No Link ECT handshake.</t>
+          <t>A15 pin 8 MGC output (D16 option A). Solder onto the factory L-Y lead. | D16: amp drives k_acc coil 85. Link only sends ACT kill on Aux 4.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>w_acc_trig</t>
+          <t>w_ac_psw_sw</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4741,48 +4737,52 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>K-ACC</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SP-AC-PSW</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>leg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A/C clutch relay coil (-)</t>
+          <t>A/C pressure sw out</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4794,17 +4794,17 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>280919-2</t>
+          <t>solder splice SP-AC-PSW</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
+          <t>OEM A/C amplifier</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>B2-M5 A/C clutch relay (k_acc) - amp A15 pin 8 sinks coil- (85); coil+ (86) fused +12 V from B2-BUS2-8</t>
+          <t>via SP-AC-PSW</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4819,26 +4819,30 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15), behind the glove box; OEM colour L-Y; EWD 1993 p.210-211; solder onto the factory lead</t>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>A15 pin 8 MGC output (D16 option A). Solder onto the factory L-Y lead. | D16: amp drives k_acc coil 85. Link only sends ACT kill on Aux 4.</t>
+          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>w_ac_psw_sw</t>
+          <t>w_tach_18</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4848,22 +4852,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-TACH</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4873,12 +4877,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>Engine speed (tacho)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4888,12 +4892,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4905,22 +4909,22 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>solder splice SP-AC-PSW</t>
+          <t>solder splice SP-TACH</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier</t>
+          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>via SP-AC-PSW</t>
+          <t>via SP-TACH</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>TACH</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -4930,7 +4934,7 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-TACH</t>
         </is>
       </c>
       <c r="V42" t="inlineStr"/>
@@ -4941,44 +4945,44 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD; OEM colour Y-R; EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell 1993 Celica component locations; solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>A/C amplifier A18 (1993: A15) pin 18, behind the glove box; OEM colour B; EWD 1993 p.211; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
+          <t>A15 pin 18 RPM input; 10-14 V average with the engine running (Mitchell 1993 Electrical). | D16: Ign 8 tacho to A15 pin 18.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>w_tach_18</t>
+          <t>w_amb_sg</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>A18</t>
+          <t>A32</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4988,12 +4992,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Engine speed (tacho)</t>
+          <t>A/C sensor common</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -5003,12 +5007,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
@@ -5020,22 +5024,22 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>solder splice SP-TACH</t>
+          <t>solder splice SP-AC-SG</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>OEM A/C amplifier A18 (1993 book: A15)</t>
+          <t>OEM auto A/C amplifier A32 pin 15 SG</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>via SP-TACH</t>
+          <t>via SP-AC-SG</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>TACH</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
@@ -5045,23 +5049,19 @@
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
+      <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr">
         <is>
-          <t>A/C amplifier A18 (1993: A15) pin 18, behind the glove box; OEM colour B; EWD 1993 p.211; solder onto the factory lead</t>
+          <t>Auto A/C amplifier A32 pin 15 SG, behind the glove box; OEM colour V-W; EWD 1993 p.211-212; solder onto the factory lead</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>A15 pin 18 RPM input; 10-14 V average with the engine running (Mitchell 1993 Electrical). | D16: Ign 8 tacho to A15 pin 18.</t>
+          <t>Cabin landing of SP-AC-SG on the amp sensor common.</t>
         </is>
       </c>
     </row>
@@ -5114,7 +5114,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>990</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -7409,7 +7409,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -9514,7 +9514,7 @@
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -9629,7 +9629,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -9740,7 +9740,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -9855,7 +9855,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -9970,7 +9970,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2820</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2820</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -10279,7 +10279,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>530</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>530</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -10616,7 +10616,7 @@
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -10834,7 +10834,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>640</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -11155,7 +11155,7 @@
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -12118,7 +12118,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -12221,7 +12221,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>3130</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -12875,7 +12875,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>680</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -12986,7 +12986,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -13089,7 +13089,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -13192,7 +13192,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -13703,7 +13703,7 @@
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -13814,7 +13814,7 @@
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -13925,7 +13925,7 @@
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -14258,7 +14258,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -14323,7 +14323,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>w_amb_sg</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -14338,12 +14338,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>A32</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>A/C sensor common</t>
+          <t>Ambient sensor return</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -14390,7 +14390,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -14400,7 +14400,7 @@
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>OEM auto A/C amplifier A32 pin 15 SG</t>
+          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
@@ -14422,12 +14422,12 @@
       <c r="W129" t="inlineStr"/>
       <c r="X129" t="inlineStr">
         <is>
-          <t>Auto A/C amplifier A32 pin 15 SG, behind the glove box; OEM colour V-W; EWD 1993 p.211-212; solder onto the factory lead</t>
+          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>Cabin landing of SP-AC-SG on the amp sensor common.</t>
+          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14484,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -14706,7 +14706,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -14809,7 +14809,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -15566,7 +15566,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -15677,7 +15677,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>820</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -18621,7 +18621,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>w_amb_sg</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">

</xml_diff>

<commit_message>
Retire the layout / schematic drawing PDFs: harnesses are built in harness.design (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$141</definedName>

</xml_diff>

<commit_message>
Retire the layout / schematic drawing PDFs: harnesses are built in harness.design (Dan 2026-11-01) (#456)
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wires" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Splices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Wires" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Connectors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Splices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spare Cavities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$141</definedName>

</xml_diff>

<commit_message>
harness.design format rules; AB-engine device pin text; reverse switch naming (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -4762,7 +4762,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>A/C pressure switch signal</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Back-up sw +12 V in</t>
+          <t>+12 V to reverse switch</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>A/C pressure switch signal</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Reverse sw +12 V out</t>
+          <t>Switched +12 V from reverse switch</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -14724,7 +14724,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -18259,7 +18259,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>

<commit_message>
harness.design format rules; AB-engine device pin text; reverse switch naming (Dan 2026-11-01) (#462)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -4762,7 +4762,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>A/C pressure switch signal</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Back-up sw +12 V in</t>
+          <t>+12 V to reverse switch</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>A/C pressure switch signal</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Reverse sw +12 V out</t>
+          <t>Switched +12 V from reverse switch</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -14724,7 +14724,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -18259,7 +18259,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch out to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>

<commit_message>
Row 171: shielded cable both sides of the firewall; device pin text; ownership audit row 182; current state refreshed (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1048,7 +1048,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1073,11 +1073,19 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -1124,7 +1132,11 @@
         </is>
       </c>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2122,7 +2134,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2132,7 +2144,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2147,11 +2159,19 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2198,7 +2218,11 @@
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2546,7 +2570,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2556,7 +2580,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2571,11 +2595,19 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2622,7 +2654,11 @@
         </is>
       </c>
       <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2653,7 +2689,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2663,7 +2699,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2678,11 +2714,19 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>CAB-FLEX-C</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2729,7 +2773,11 @@
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); red and yellow cores unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2863,7 +2911,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2873,7 +2921,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2888,11 +2936,19 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2939,7 +2995,11 @@
         </is>
       </c>
       <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3283,7 +3343,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3293,7 +3353,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3308,11 +3368,19 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -3355,7 +3423,11 @@
       </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3695,7 +3767,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3705,7 +3777,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3720,11 +3792,19 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-WHITE</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
           <t>3-1447221-3</t>
@@ -3767,7 +3847,11 @@
       </c>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4111,7 +4195,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4121,7 +4205,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4136,11 +4220,19 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-WHITE</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr">
         <is>
           <t>3-1447221-3</t>
@@ -4183,7 +4275,11 @@
       </c>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4433,7 +4529,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Ambient temp signal</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -5099,7 +5195,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>+5 V (sensor 2)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -5214,7 +5310,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Gnd (sensor 2)</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -5329,7 +5425,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
+          <t>Signal 2 (sub)</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5444,7 +5540,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
+          <t>+5 V (sensor 1)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5559,7 +5655,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
+          <t>Gnd (sensor 1)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5674,7 +5770,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>Signal 1 (main)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5784,7 +5880,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -5794,7 +5890,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5804,16 +5900,24 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O50" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -5860,7 +5964,11 @@
         </is>
       </c>
       <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5998,7 +6106,7 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -6008,7 +6116,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -6018,16 +6126,24 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O52" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6074,7 +6190,11 @@
         </is>
       </c>
       <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6641,7 +6761,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Gnd IAT/TPS/coolant</t>
+          <t>Gnd to intake temp, throttle sensor, coolant temp</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6743,7 +6863,7 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -6763,16 +6883,24 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O59" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6819,7 +6947,11 @@
         </is>
       </c>
       <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6850,7 +6982,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -6860,7 +6992,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -6870,16 +7002,24 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6926,7 +7066,11 @@
         </is>
       </c>
       <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6957,7 +7101,7 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -6967,7 +7111,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6977,16 +7121,24 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O61" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -7033,7 +7185,11 @@
         </is>
       </c>
       <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7069,7 +7225,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Gnd flex + MAP</t>
+          <t>Gnd to flex fuel, MAP sensor</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7176,7 +7332,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Gnd oil/clnt/temps</t>
+          <t>Gnd to oil pressure, coolant pressure, oil temp, charge temp</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7283,7 +7439,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Gnd fuel press + VSS</t>
+          <t>Gnd to fuel pressure, gearbox speed</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7722,7 +7878,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -7732,14 +7888,10 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
           <t>630</t>
@@ -7747,11 +7899,19 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>CAB-FLEX-C</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O68" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -7798,7 +7958,11 @@
         </is>
       </c>
       <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7833,7 +7997,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -7843,14 +8007,10 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>630</t>
@@ -7858,11 +8018,19 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O69" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -7909,7 +8077,11 @@
         </is>
       </c>
       <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7944,7 +8116,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -7954,14 +8126,10 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>630</t>
@@ -7969,11 +8137,19 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O70" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8016,7 +8192,11 @@
       </c>
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8051,7 +8231,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -8061,14 +8241,10 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>630</t>
@@ -8076,11 +8252,19 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O71" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8127,7 +8311,11 @@
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8162,7 +8350,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -8172,7 +8360,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -8182,16 +8370,24 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O72" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8238,7 +8434,11 @@
         </is>
       </c>
       <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8273,7 +8473,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -8283,7 +8483,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -8293,16 +8493,24 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O73" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8349,7 +8557,11 @@
         </is>
       </c>
       <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8384,7 +8596,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -8394,14 +8606,10 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>630</t>
@@ -8409,11 +8617,19 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O74" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8460,7 +8676,11 @@
         </is>
       </c>
       <c r="X74" t="inlineStr"/>
-      <c r="Y74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8709,7 +8929,7 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -8719,7 +8939,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8729,16 +8949,24 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O77" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8785,7 +9013,11 @@
         </is>
       </c>
       <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8820,7 +9052,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -8830,14 +9062,10 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>630</t>
@@ -8845,11 +9073,19 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O78" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8892,7 +9128,11 @@
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8927,7 +9167,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -8937,14 +9177,10 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>630</t>
@@ -8952,11 +9188,19 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O79" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -9005,7 +9249,7 @@
       <c r="X79" t="inlineStr"/>
       <c r="Y79" t="inlineStr">
         <is>
-          <t>build (R30): this drain is the one crimped into A7</t>
+          <t>build (R30): this drain is the one crimped into A7; cable screen: firewall pin to the shield splice</t>
         </is>
       </c>
     </row>
@@ -9622,7 +9866,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Back-up lamp +12 V</t>
+          <t>+12 V to reverse lamps</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -12959,7 +13203,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Fuel lvl pull-up</t>
+          <t>Fuel level pull-up</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -13054,7 +13298,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>+5 V fuel lvl pullup</t>
+          <t>+5 V to fuel level pull-up</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -13256,7 +13500,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Lock-sensor input (modified tacho)</t>
+          <t>Lock sensor signal (modified tacho)</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -14025,7 +14269,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>A/C pressure switch signal</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -14140,7 +14384,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Ambient sensor return</t>
+          <t>Gnd</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -14358,7 +14602,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>CSB3 + opto ground</t>
+          <t>Gnd to CSB3, opto board</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -18106,11 +18350,11 @@
         <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>4.15</v>
+        <v>1.56</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>w_drain_ecu_a (20 AWG), w_shd_a_aps (20 AWG), w_shd_a_wsf (20 AWG), w_shc_crank (20 AWG), w_shc_cam (20 AWG), w_shc_turbo (20 AWG), w_shc_flex (20 AWG), w_shc_etbs (20 AWG)</t>
+          <t>w_drain_ecu_a (20 AWG), w_shd_a_aps (20 AWG), w_shd_a_wsf (20 AWG), w_shc_crank (screen AWG), w_shc_cam (screen AWG), w_shc_turbo (screen AWG), w_shc_flex (screen AWG), w_shc_etbs (screen AWG)</t>
         </is>
       </c>
     </row>
@@ -18304,11 +18548,11 @@
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>2.08</v>
+        <v>1.04</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>w_shc_knock1 (20 AWG), w_shc_etbm (20 AWG), w_drain_ecu_b (20 AWG), w_shd_b_wsr (20 AWG)</t>
+          <t>w_shc_knock1 (screen AWG), w_shc_etbm (screen AWG), w_drain_ecu_b (20 AWG), w_shd_b_wsr (20 AWG)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Row 171: shielded cable both sides of the firewall; device pin text; ownership audit row 182; current state refreshed (Dan 2026-11-01) (#463)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -1048,7 +1048,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1073,11 +1073,19 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -1124,7 +1132,11 @@
         </is>
       </c>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2122,7 +2134,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2132,7 +2144,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2147,11 +2159,19 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2198,7 +2218,11 @@
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2546,7 +2570,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2556,7 +2580,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2571,11 +2595,19 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2622,7 +2654,11 @@
         </is>
       </c>
       <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2653,7 +2689,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2663,7 +2699,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2678,11 +2714,19 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>CAB-FLEX-C</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2729,7 +2773,11 @@
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); red and yellow cores unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2863,7 +2911,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2873,7 +2921,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2888,11 +2936,19 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -2939,7 +2995,11 @@
         </is>
       </c>
       <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3283,7 +3343,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3293,7 +3353,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3308,11 +3368,19 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>3-1447221-4</t>
@@ -3355,7 +3423,11 @@
       </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3695,7 +3767,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3705,7 +3777,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3720,11 +3792,19 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-WHITE</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
           <t>3-1447221-3</t>
@@ -3767,7 +3847,11 @@
       </c>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4111,7 +4195,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4121,7 +4205,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4136,11 +4220,19 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-WHITE</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr">
         <is>
           <t>3-1447221-3</t>
@@ -4183,7 +4275,11 @@
       </c>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4433,7 +4529,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Ambient temp signal</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -5099,7 +5195,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>+5 V (sensor 2)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -5214,7 +5310,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Gnd (sensor 2)</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -5329,7 +5425,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
+          <t>Signal 2 (sub)</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5444,7 +5540,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
+          <t>+5 V (sensor 1)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5559,7 +5655,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
+          <t>Gnd (sensor 1)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5674,7 +5770,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>Signal 1 (main)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5784,7 +5880,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -5794,7 +5890,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5804,16 +5900,24 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O50" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -5860,7 +5964,11 @@
         </is>
       </c>
       <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171); yellow core unused in the cabin: cut back and sealed under heat shrink at both ends</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5998,7 +6106,7 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -6008,7 +6116,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -6018,16 +6126,24 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O52" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6074,7 +6190,11 @@
         </is>
       </c>
       <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6641,7 +6761,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Gnd IAT/TPS/coolant</t>
+          <t>Gnd to intake temp, throttle sensor, coolant temp</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6743,7 +6863,7 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -6763,16 +6883,24 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O59" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6819,7 +6947,11 @@
         </is>
       </c>
       <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6850,7 +6982,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -6860,7 +6992,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -6870,16 +7002,24 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -6926,7 +7066,11 @@
         </is>
       </c>
       <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6957,7 +7101,7 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -6967,7 +7111,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6977,16 +7121,24 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O61" t="inlineStr">
         <is>
           <t>0462-201-16141</t>
@@ -7033,7 +7185,11 @@
         </is>
       </c>
       <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7069,7 +7225,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Gnd flex + MAP</t>
+          <t>Gnd to flex fuel, MAP sensor</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7176,7 +7332,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Gnd oil/clnt/temps</t>
+          <t>Gnd to oil pressure, coolant pressure, oil temp, charge temp</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7283,7 +7439,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Gnd fuel press + VSS</t>
+          <t>Gnd to fuel pressure, gearbox speed</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7722,7 +7878,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -7732,14 +7888,10 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
           <t>630</t>
@@ -7747,11 +7899,19 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>CAB-FLEX-C</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O68" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -7798,7 +7958,11 @@
         </is>
       </c>
       <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7833,7 +7997,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -7843,14 +8007,10 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>630</t>
@@ -7858,11 +8018,19 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>CAB-ETBS-C</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>55A1841-20-2/4/5/6-9</t>
+        </is>
+      </c>
       <c r="O69" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -7909,7 +8077,11 @@
         </is>
       </c>
       <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7944,7 +8116,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -7954,14 +8126,10 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>630</t>
@@ -7969,11 +8137,19 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>CAB-ETBM-C</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>55A1821-18-2/0-9</t>
+        </is>
+      </c>
       <c r="O70" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8016,7 +8192,11 @@
       </c>
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8051,7 +8231,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -8061,14 +8241,10 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>630</t>
@@ -8076,11 +8252,19 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>CAB-TURBO-C</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O71" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8127,7 +8311,11 @@
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8162,7 +8350,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -8172,7 +8360,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -8182,16 +8370,24 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O72" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8238,7 +8434,11 @@
         </is>
       </c>
       <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8273,7 +8473,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -8283,7 +8483,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -8293,16 +8493,24 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O73" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8349,7 +8557,11 @@
         </is>
       </c>
       <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8384,7 +8596,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -8394,14 +8606,10 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>630</t>
@@ -8409,11 +8617,19 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>CAB-CAM-C</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>55A1831-20-2/4/6-9</t>
+        </is>
+      </c>
       <c r="O74" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8460,7 +8676,11 @@
         </is>
       </c>
       <c r="X74" t="inlineStr"/>
-      <c r="Y74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8709,7 +8929,7 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>wire</t>
+          <t>core</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -8719,7 +8939,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8729,16 +8949,24 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>630</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLUE</t>
-        </is>
-      </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O77" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8785,7 +9013,11 @@
         </is>
       </c>
       <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>same Spec 55 cable both sides of the firewall (B14, row 171)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8820,7 +9052,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -8830,14 +9062,10 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>630</t>
@@ -8845,11 +9073,19 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>CAB-KNOCK1-C</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O78" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -8892,7 +9128,11 @@
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>cable screen: firewall pin to the shield splice</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8927,7 +9167,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>leg</t>
+          <t>leg core</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -8937,14 +9177,10 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>630</t>
@@ -8952,11 +9188,19 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>CAB-CRANK-C</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>55A1821-20-6/9-9</t>
+        </is>
+      </c>
       <c r="O79" t="inlineStr">
         <is>
           <t>0460-202-1631</t>
@@ -9005,7 +9249,7 @@
       <c r="X79" t="inlineStr"/>
       <c r="Y79" t="inlineStr">
         <is>
-          <t>build (R30): this drain is the one crimped into A7</t>
+          <t>build (R30): this drain is the one crimped into A7; cable screen: firewall pin to the shield splice</t>
         </is>
       </c>
     </row>
@@ -9622,7 +9866,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Back-up lamp +12 V</t>
+          <t>+12 V to reverse lamps</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -12959,7 +13203,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Fuel lvl pull-up</t>
+          <t>Fuel level pull-up</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -13054,7 +13298,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>+5 V fuel lvl pullup</t>
+          <t>+5 V to fuel level pull-up</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -13256,7 +13500,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Lock-sensor input (modified tacho)</t>
+          <t>Lock sensor signal (modified tacho)</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -14025,7 +14269,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>A/C pressure switch signal</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -14140,7 +14384,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Ambient sensor return</t>
+          <t>Gnd</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -14358,7 +14602,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>CSB3 + opto ground</t>
+          <t>Gnd to CSB3, opto board</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -18106,11 +18350,11 @@
         <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>4.15</v>
+        <v>1.56</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>w_drain_ecu_a (20 AWG), w_shd_a_aps (20 AWG), w_shd_a_wsf (20 AWG), w_shc_crank (20 AWG), w_shc_cam (20 AWG), w_shc_turbo (20 AWG), w_shc_flex (20 AWG), w_shc_etbs (20 AWG)</t>
+          <t>w_drain_ecu_a (20 AWG), w_shd_a_aps (20 AWG), w_shd_a_wsf (20 AWG), w_shc_crank (screen AWG), w_shc_cam (screen AWG), w_shc_turbo (screen AWG), w_shc_flex (screen AWG), w_shc_etbs (screen AWG)</t>
         </is>
       </c>
     </row>
@@ -18304,11 +18548,11 @@
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>2.08</v>
+        <v>1.04</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>w_shc_knock1 (20 AWG), w_shc_etbm (20 AWG), w_drain_ecu_b (20 AWG), w_shd_b_wsr (20 AWG)</t>
+          <t>w_shc_knock1 (screen AWG), w_shc_etbm (screen AWG), w_drain_ecu_b (20 AWG), w_shd_b_wsr (20 AWG)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harness ownership: one plug = one harness, 22 wires moved; pin chart devices-by-harness page; row 182 closed (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Connectors'!$A$1:$I$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Splices'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$61</definedName>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y140"/>
+  <dimension ref="A1:Y141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>ST185-AntiTheft</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4380,7 +4380,7 @@
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on ECU-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on ECU-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm); harness ownership (Dan 2026-11-01): was AntiTheft via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -9361,7 +9361,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>ST185-AB-engine wc_h_lam_be at DRB102-ENGINE 79, to splice SP-CANH-LAM; SP-CANH also joins ST185-CAN</t>
+          <t>ST185-AB-engine wc_h_lam_be at DRB102-ENGINE 79, to splice SP-CANH-LAM; SP-CANH also joins ST185-CAN, ST185-CSB3</t>
         </is>
       </c>
       <c r="W80" t="inlineStr"/>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>ST185-AB-engine wc_l_lam_be at DRB102-ENGINE 80, to splice SP-CANL-LAM; SP-CANL also joins ST185-CAN</t>
+          <t>ST185-AB-engine wc_l_lam_be at DRB102-ENGINE 80, to splice SP-CANL-LAM; SP-CANL also joins ST185-CAN, ST185-CSB3</t>
         </is>
       </c>
       <c r="W81" t="inlineStr"/>
@@ -11646,7 +11646,7 @@
       </c>
       <c r="T101" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U101" t="inlineStr">
@@ -11663,7 +11663,7 @@
       <c r="X101" t="inlineStr"/>
       <c r="Y101" t="inlineStr">
         <is>
-          <t>POWER box (glove box) relay R2 EFI main, pin 85 | owner proposed: longer half (drawn today as w76 on ECU-cabin, 370 mm; w76_cp on CabinPower, 400 mm)</t>
+          <t>POWER box (glove box) relay R2 EFI main, pin 85 | owner proposed: longer half (drawn today as w76 on ECU-cabin, 370 mm; w76_cp on CabinPower, 400 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -11864,7 +11864,7 @@
       </c>
       <c r="T103" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U103" t="inlineStr">
@@ -11881,7 +11881,7 @@
       <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) relay M14 ETB power, pin 85 | owner proposed: longer half (drawn today as w81 on ECU-cabin, 380 mm; w81_cp on CabinPower, 400 mm)</t>
+          <t>LOGIC box (glove box) relay M14 ETB power, pin 85 | owner proposed: longer half (drawn today as w81 on ECU-cabin, 380 mm; w81_cp on CabinPower, 400 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="T104" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U104" t="inlineStr">
@@ -11984,7 +11984,7 @@
       <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w82_ac on CabinPower, 400 mm; w82 on ECU-cabin, 340 mm)</t>
+          <t>owner proposed: longer half (drawn today as w82_ac on CabinPower, 400 mm; w82 on ECU-cabin, 340 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12391,7 +12391,7 @@
       </c>
       <c r="T108" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U108" t="inlineStr">
@@ -12408,7 +12408,7 @@
       <c r="X108" t="inlineStr"/>
       <c r="Y108" t="inlineStr">
         <is>
-          <t>CAN-Lambda +12 V | CAN-Lambda +12 V | owner proposed: longer half (drawn today as w_lam12_cp on CabinPower, 250 mm; w_lam12_bc on ECU-cabin, 120 mm)</t>
+          <t>CAN-Lambda +12 V | CAN-Lambda +12 V | owner proposed: longer half (drawn today as w_lam12_cp on CabinPower, 250 mm; w_lam12_bc on ECU-cabin, 120 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12712,7 @@
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
@@ -12733,7 +12733,7 @@
       <c r="X111" t="inlineStr"/>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse COP 10A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse COP 10A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12823,7 +12823,7 @@
       </c>
       <c r="T112" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U112" t="inlineStr">
@@ -12844,7 +12844,7 @@
       <c r="X112" t="inlineStr"/>
       <c r="Y112" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse INJ 7.5A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse INJ 7.5A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -13683,89 +13683,85 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>cab_aps1_sh</t>
+          <t>w_strl_c</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>NC, floats</t>
+          <t>RB4</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>drain</t>
+          <t>wire</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Starter solenoid S</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Shield</t>
-        </is>
-      </c>
-      <c r="J121" t="inlineStr"/>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>(cable core)</t>
-        </is>
-      </c>
-      <c r="M121" t="inlineStr">
-        <is>
-          <t>CAB-APS1</t>
-        </is>
-      </c>
-      <c r="N121" t="inlineStr">
-        <is>
-          <t>55A1831-20-2/4/6-9</t>
-        </is>
-      </c>
-      <c r="O121" t="inlineStr"/>
+          <t>J1128-TXL-12-RED</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>crimp butt splice into the factory lead</t>
+        </is>
+      </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>solder splice SP-SHIELD-A-APS</t>
+          <t>0460-220-1231</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>cab_aps1 screen (floats at the device end)</t>
+          <t>OEM R/B No.4 starter relay pin 4 (RH kick), starter out</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>via SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13775,26 +13771,30 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS</t>
-        </is>
-      </c>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
-      <c r="X121" t="inlineStr"/>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_strl_e at DRB102-ENGINE 3, to STARTER-TRIGGER 1</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>R/B No.4 starter relay pin 4, RH kick; OEM colour B; EWD 1993 p.66; crimp butt splice into the factory lead at R/B No.4 pin 4</t>
+        </is>
+      </c>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>Screen floats at this end: cut back and seal under heat-shrink | screen floats at the far end; pedal branch length estimated from OEM body dimensions + 10 % (990 mm ECU-A</t>
+          <t>OEM starter relay output (was EB1-2). New wire to the starter S terminal. | (firewall bulkhead, RH) | Starter S crosses the firewall on its own DRB102 size-12 cavity (Dan 2026-10-27); 12 AWG: the DRB size-12 contact takes 12-14 AWG, solenoid S draw is brief, OEM lead is lighter; harness ownership (Dan 2026-11-01): was CabinPower</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>cab_aps_sh</t>
+          <t>cab_aps1_sh</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -13829,7 +13829,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>CAB-APS2</t>
+          <t>CAB-APS1</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>cab_aps2 screen (floats at the device end)</t>
+          <t>cab_aps1 screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -13905,7 +13905,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_sh_ac</t>
+          <t>cab_aps_sh</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -13940,7 +13940,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -13951,7 +13951,7 @@
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -13961,33 +13961,33 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>CAB-FSPUR-FR-AC</t>
+          <t>CAB-APS2</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>55A1811-20-9-9CS2275</t>
+          <t>55A1831-20-2/4/6-9</t>
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
-          <t>solder splice SP-SHIELD-A-WSF</t>
+          <t>solder splice SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac screen (floats at the device end)</t>
+          <t>cab_aps2 screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>via SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>via SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
@@ -13997,36 +13997,36 @@
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF</t>
+          <t>SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
       <c r="Y123" t="inlineStr">
         <is>
-          <t>Screen floats at this end: cut back and seal under heat-shrink | tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+          <t>Screen floats at this end: cut back and seal under heat-shrink | screen floats at the far end; pedal branch length estimated from OEM body dimensions + 10 % (990 mm ECU-A</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>w19</t>
+          <t>cab_fspur_fr_sh_ac</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>legs of SP-8V</t>
+          <t>NC, floats</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -14036,69 +14036,69 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>SP-8V</t>
+          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>drain</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>+8 V sensor supply</t>
+          <t>FR wheel spd shield</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>solder splice</t>
-        </is>
-      </c>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>CAB-FSPUR-FR-AC</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>55A1811-20-9-9CS2275</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>solder splice SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-8V: +8 V supply, cam sensor + gearbox speed sensor only (ECU A6)</t>
+          <t>cab_fspur_fr_ac screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>via SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>8V</t>
+          <t>WSSF</t>
         </is>
       </c>
       <c r="T124" t="inlineStr">
@@ -14108,27 +14108,31 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>SP-8V</t>
+          <t>SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>dash branch (front WS inline)</t>
         </is>
       </c>
       <c r="X124" t="inlineStr"/>
-      <c r="Y124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>Screen floats at this end: cut back and seal under heat-shrink | tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>w_a5_pin</t>
+          <t>w19</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>legs of SP-A5</t>
+          <t>legs of SP-8V</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -14143,12 +14147,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>SP-A5</t>
+          <t>SP-8V</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -14158,17 +14162,17 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
+          <t>+8 V sensor supply</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -14178,7 +14182,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-RED</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="M125" t="inlineStr"/>
@@ -14190,12 +14194,12 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
+          <t>ECU splice point - SP-8V: +8 V supply, cam sensor + gearbox speed sensor only (ECU A6)</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -14205,7 +14209,7 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -14215,7 +14219,7 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>SP-A5</t>
+          <t>SP-8V</t>
         </is>
       </c>
       <c r="V125" t="inlineStr"/>
@@ -14225,21 +14229,17 @@
         </is>
       </c>
       <c r="X125" t="inlineStr"/>
-      <c r="Y125" t="inlineStr">
-        <is>
-          <t>ECU main +12 V | ECU main +12 V</t>
-        </is>
-      </c>
+      <c r="Y125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>w_ac_psw_in</t>
+          <t>w_a5_pin</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>legs of SP-AC-PSW</t>
+          <t>legs of SP-A5</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -14249,17 +14249,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-A5</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -14269,27 +14269,27 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="M126" t="inlineStr"/>
@@ -14301,22 +14301,22 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the switch's </t>
+          <t>3-1447221-3</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>At A/C amp - SP-AC-PSW: A/C pressure switch output</t>
+          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>OEM A5, factory Y-R lead</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SW12</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14326,35 +14326,31 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-A5</t>
         </is>
       </c>
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="X126" t="inlineStr">
-        <is>
-          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo); OEM colour Y-R (factory wiring; new wire here); EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R); new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
-        </is>
-      </c>
+          <t>at ECU-A plug</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr"/>
       <c r="Y126" t="inlineStr">
         <is>
-          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152. | owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on ECU-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
+          <t>ECU main +12 V | ECU main +12 V</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>w_amb_rtn</t>
+          <t>w_ac_psw_in</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>legs of SP-AC-SG</t>
+          <t>legs of SP-AC-PSW</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -14364,17 +14360,17 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -14384,7 +14380,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Gnd</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -14399,12 +14395,12 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-YELLOW</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="M127" t="inlineStr"/>
@@ -14416,22 +14412,22 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
+          <t xml:space="preserve">new-wire run terminated at the switch's </t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>SP-AC-SG - cabin A/C sensor common (replaces E10; A32-15, A24-3, A21, A18-2 stay factory)</t>
+          <t>At A/C amp - SP-AC-PSW: A/C pressure switch output</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
+          <t>OEM A5, factory Y-R lead</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14441,31 +14437,35 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="V127" t="inlineStr"/>
-      <c r="W127" t="inlineStr"/>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo); OEM colour Y-R (factory wiring; new wire here); EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R); new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
         <is>
-          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152. | owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on ECU-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>w_trig2_pin</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>legs of SP-CAM</t>
+          <t>legs of SP-AC-SG</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -14475,17 +14475,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>SP-CAM</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -14495,12 +14495,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Cam sensor signal</t>
+          <t>Gnd</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -14510,12 +14510,12 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="M128" t="inlineStr"/>
@@ -14527,22 +14527,22 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>At the ECU plugs - SP-CAM: cam signal + 1.8k pull-up to +8V</t>
+          <t>SP-AC-SG - cabin A/C sensor common (replaces E10; A32-15, A24-3, A21, A18-2 stay factory)</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
@@ -14552,27 +14552,31 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>SP-CAM</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="V128" t="inlineStr"/>
-      <c r="W128" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
-      <c r="X128" t="inlineStr"/>
-      <c r="Y128" t="inlineStr"/>
+      <c r="W128" t="inlineStr"/>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>w_csbg_ac</t>
+          <t>w_trig2_pin</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>legs of SP-CSB-GND</t>
+          <t>legs of SP-CAM</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -14582,17 +14586,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>SP-CSB-GND</t>
+          <t>SP-CAM</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -14602,12 +14606,12 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Gnd to CSB3, opto board</t>
+          <t>Cam sensor signal</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14617,12 +14621,12 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLACK</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M129" t="inlineStr"/>
@@ -14634,22 +14638,22 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>CSB3 ground splice - CSB3 pin 2, opto board COM and stalk ground</t>
+          <t>At the ECU plugs - SP-CAM: cam signal + 1.8k pull-up to +8V</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14659,35 +14663,27 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>SP-CSB-GND</t>
-        </is>
-      </c>
-      <c r="V129" t="inlineStr">
-        <is>
-          <t>SP-CSB-GND also joins ST185-CSB3</t>
-        </is>
-      </c>
+          <t>SP-CAM</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr">
         <is>
-          <t>glove-box POWER box to the CSB3 branch</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X129" t="inlineStr"/>
-      <c r="Y129" t="inlineStr">
-        <is>
-          <t>M8 ring lug on the POWER box battery-negative bar (R213: CSB3, opto board and cruise ladder never on chassis or the ECU ground) | (CSB3 loom, under centre cluster) | est length; runs with the CSB3 +12 V (w_csb12, LOGIC CSB 5A) (R217)</t>
-        </is>
-      </c>
+      <c r="Y129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>w_fl_sig_pin</t>
+          <t>w_csbg_ac</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>legs of SP-FUEL-LVL</t>
+          <t>legs of SP-CSB-GND</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -14697,17 +14693,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL</t>
+          <t>SP-CSB-GND</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -14717,12 +14713,12 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Fuel level signal</t>
+          <t>Gnd to CSB3, opto board</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14732,12 +14728,12 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="M130" t="inlineStr"/>
@@ -14749,22 +14745,22 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL - fuel sender signal + 470R pull-up to ECU-B B24</t>
+          <t>CSB3 ground splice - CSB3 pin 2, opto board COM and stalk ground</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>FLVL</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14774,23 +14770,35 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL</t>
-        </is>
-      </c>
-      <c r="V130" t="inlineStr"/>
-      <c r="W130" t="inlineStr"/>
+          <t>SP-CSB-GND</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>SP-CSB-GND also joins ST185-CSB3</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>glove-box POWER box to the CSB3 branch</t>
+        </is>
+      </c>
       <c r="X130" t="inlineStr"/>
-      <c r="Y130" t="inlineStr"/>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>M8 ring lug on the POWER box battery-negative bar (R213: CSB3, opto board and cruise ladder never on chassis or the ECU ground) | (CSB3 loom, under centre cluster) | est length; runs with the CSB3 +12 V (w_csb12, LOGIC CSB 5A) (R217)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>w66</t>
+          <t>w_fl_sig_pin</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>legs of SP-GND-ECU</t>
+          <t>legs of SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -14800,17 +14808,17 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>24</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>SP-GND-ECU</t>
+          <t>SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -14820,27 +14828,27 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>ECU power ground</t>
+          <t>Fuel level signal</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>J1128-TXL-10-BLACK</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M131" t="inlineStr"/>
@@ -14852,22 +14860,22 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-GND-ECU: ECU power ground (A25 A34 B25 B34) to the NEG bar</t>
+          <t>SP-FUEL-LVL - fuel sender signal + 470R pull-up to ECU-B B24</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>GND</t>
+          <t>FLVL</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14877,31 +14885,23 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>SP-GND-ECU</t>
+          <t>SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="V131" t="inlineStr"/>
-      <c r="W131" t="inlineStr">
-        <is>
-          <t>ECU to the glove-box POWER box</t>
-        </is>
-      </c>
+      <c r="W131" t="inlineStr"/>
       <c r="X131" t="inlineStr"/>
-      <c r="Y131" t="inlineStr">
-        <is>
-          <t>M8 ring lug on the POWER box battery-negative bar (R216): the ECU grounds only, nothing else | est length; the ONE ECU ground return (DECISIONS R216)</t>
-        </is>
-      </c>
+      <c r="Y131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>w_rev_sw_c</t>
+          <t>w66</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>legs of SP-REV</t>
+          <t>legs of SP-GND-ECU</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -14911,17 +14911,17 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>DRB102-CABIN</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>SP-REV</t>
+          <t>SP-GND-ECU</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -14931,27 +14931,27 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Switched +12 V from reverse switch</t>
+          <t>ECU power ground</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>J1128-TXL-16-YELLOW</t>
+          <t>J1128-TXL-10-BLACK</t>
         </is>
       </c>
       <c r="M132" t="inlineStr"/>
@@ -14963,22 +14963,22 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>0460-202-1631</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>ECU splice point - SP-GND-ECU: ECU power ground (A25 A34 B25 B34) to the NEG bar</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>DRB102 receptacle (RH firewall)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14988,31 +14988,31 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>SP-REV</t>
-        </is>
-      </c>
-      <c r="V132" t="inlineStr">
-        <is>
-          <t>ST185-AB-engine w_sw7_e at DRB102-ENGINE 78, to REV-SW 1</t>
-        </is>
-      </c>
-      <c r="W132" t="inlineStr"/>
+          <t>SP-GND-ECU</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr"/>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>ECU to the glove-box POWER box</t>
+        </is>
+      </c>
       <c r="X132" t="inlineStr"/>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>Circuit 11: switch out tapped to opto IN2; lamps stay on the factory IG2-13 run.</t>
+          <t>M8 ring lug on the POWER box battery-negative bar (R216): the ECU grounds only, nothing else | est length; the ONE ECU ground return (DECISIONS R216)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>w_drain_ecu_a</t>
+          <t>w_rev_sw_c</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A</t>
+          <t>legs of SP-REV</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -15022,17 +15022,17 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>78</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A</t>
+          <t>SP-REV</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -15042,27 +15042,27 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Shield drain</t>
+          <t>Switched +12 V from reverse switch</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="M133" t="inlineStr"/>
@@ -15074,22 +15074,22 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>0460-202-1631</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>SHLD</t>
+          <t>REV</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -15099,31 +15099,31 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A</t>
-        </is>
-      </c>
-      <c r="V133" t="inlineStr"/>
-      <c r="W133" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
+          <t>SP-REV</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_sw7_e at DRB102-ENGINE 78, to REV-SW 1</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr"/>
       <c r="X133" t="inlineStr"/>
       <c r="Y133" t="inlineStr">
         <is>
-          <t>build (R30): the crank drain is the one crimped into A7; the other drains are soldered onto it 6 mm behind the plug</t>
+          <t>Circuit 11: switch out tapped to opto IN2; lamps stay on the factory IG2-13 run.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>w_shd_a_aps</t>
+          <t>w_drain_ecu_a</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A-APS</t>
+          <t>legs of SP-SHIELD-A</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -15133,22 +15133,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -15168,7 +15168,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -15185,17 +15185,17 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>solder splice</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
+          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
@@ -15210,27 +15210,31 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS / SP-SHIELD-A</t>
+          <t>SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V134" t="inlineStr"/>
-      <c r="W134" t="inlineStr"/>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>at ECU-A plug</t>
+        </is>
+      </c>
       <c r="X134" t="inlineStr"/>
       <c r="Y134" t="inlineStr">
         <is>
-          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+          <t>build (R30): the crank drain is the one crimped into A7; the other drains are soldered onto it 6 mm behind the plug</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>w_shd_a_wsf</t>
+          <t>w_shd_a_aps</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A-WSF</t>
+          <t>legs of SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -15250,7 +15254,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -15275,7 +15279,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -15297,7 +15301,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
+          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -15317,7 +15321,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF / SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS / SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V135" t="inlineStr"/>
@@ -15332,12 +15336,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>w_drain_ecu_b</t>
+          <t>w_shd_a_wsf</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B</t>
+          <t>legs of SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -15347,27 +15351,27 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>legs of SP-SHIELD-A</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B</t>
+          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>link</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Shield drain B</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -15382,7 +15386,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -15399,17 +15403,17 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
+          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
@@ -15424,23 +15428,27 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B</t>
+          <t>SP-SHIELD-A-WSF / SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V136" t="inlineStr"/>
       <c r="W136" t="inlineStr"/>
       <c r="X136" t="inlineStr"/>
-      <c r="Y136" t="inlineStr"/>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>w_shd_b_wsr</t>
+          <t>w_drain_ecu_b</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B-WSR</t>
+          <t>legs of SP-SHIELD-B</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -15450,22 +15458,22 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B-WSR &gt; SP-SHIELD-B</t>
+          <t>SP-SHIELD-B</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -15485,7 +15493,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -15502,17 +15510,17 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>solder splice</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>At the rear WS inline - SP-SHIELD-B-WSR: rear wheel-speed drains</t>
+          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
@@ -15527,27 +15535,23 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B-WSR / SP-SHIELD-B</t>
+          <t>SP-SHIELD-B</t>
         </is>
       </c>
       <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr"/>
-      <c r="Y137" t="inlineStr">
-        <is>
-          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
-        </is>
-      </c>
+      <c r="Y137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>w78</t>
+          <t>w_shd_b_wsr</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>legs of SP-SW12</t>
+          <t>legs of SP-SHIELD-B-WSR</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -15557,7 +15561,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>legs of SP-A5</t>
+          <t>legs of SP-SHIELD-B</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -15567,7 +15571,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>SP-SW12 &gt; SP-A5</t>
+          <t>SP-SHIELD-B-WSR &gt; SP-SHIELD-B</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -15577,27 +15581,27 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
+          <t>Shield drain B</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-RED</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
@@ -15614,17 +15618,17 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-SW12: switched +12 V (LOGIC SW12)</t>
+          <t>At the rear WS inline - SP-SHIELD-B-WSR: rear wheel-speed drains</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
+          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15634,26 +15638,22 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>SP-SW12 / SP-A5</t>
+          <t>SP-SHIELD-B-WSR / SP-SHIELD-B</t>
         </is>
       </c>
       <c r="V138" t="inlineStr"/>
-      <c r="W138" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
+      <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr"/>
       <c r="Y138" t="inlineStr">
         <is>
-          <t>ECU main +12 V | ECU main +12 V</t>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>w_rail_sp_sw12_c</t>
+          <t>w78</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -15668,27 +15668,27 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>DRB102-CABIN</t>
+          <t>legs of SP-A5</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>SP-SW12</t>
+          <t>SP-SW12 &gt; SP-A5</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>link</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -15703,7 +15703,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>0460-202-1631</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>DRB102 receptacle (RH firewall)</t>
+          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
@@ -15745,35 +15745,31 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>SP-SW12</t>
-        </is>
-      </c>
-      <c r="V139" t="inlineStr">
-        <is>
-          <t>ST185-AB-engine w_rail_sp_sw12_e at DRB102-ENGINE 30, to splice SP-SW12-ENG</t>
-        </is>
-      </c>
+          <t>SP-SW12 / SP-A5</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr">
         <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X139" t="inlineStr"/>
       <c r="Y139" t="inlineStr">
         <is>
-          <t>+12 V boost + flex | +12 V boost + flex</t>
+          <t>ECU main +12 V | ECU main +12 V</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>w_tach</t>
+          <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>legs of SP-TACH</t>
+          <t>legs of SP-SW12</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -15783,17 +15779,17 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-SW12</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -15803,27 +15799,27 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Engine speed (tacho)</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="M140" t="inlineStr"/>
@@ -15835,22 +15831,22 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>0460-202-1631</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>SP-TACH - Ign 8 tacho to A15 pin 18 and 4.7k lock-sensor tap</t>
+          <t>ECU splice point - SP-SW12: switched +12 V (LOGIC SW12)</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>TACH</t>
+          <t>SW12</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15860,24 +15856,139 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
-        </is>
-      </c>
-      <c r="V140" t="inlineStr"/>
+          <t>SP-SW12</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_rail_sp_sw12_e at DRB102-ENGINE 30, to splice SP-SW12-ENG</t>
+        </is>
+      </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
       <c r="Y140" t="inlineStr">
         <is>
+          <t>+12 V boost + flex | +12 V boost + flex</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>w_tach</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>legs of SP-TACH</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>ECU-B</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>SP-TACH</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>trunk</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Engine speed (tacho)</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>J1128-TXL-20-WHITE</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>solder splice</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>3-1447221-4</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>SP-TACH - Ign 8 tacho to A15 pin 18 and 4.7k lock-sensor tap</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>TACH</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>SP-TACH</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr"/>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr">
+        <is>
           <t>Ign 8 (ECU-B 10) tacho. Split at SP-TACH: pin 18 plus 4.7k to pin 9 (OPEN-ITEMS History 2026-10-21 N61).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y140"/>
+  <autoFilter ref="A1:Y141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16278,7 +16389,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H9" t="n">
         <v>37</v>
@@ -17144,11 +17255,11 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t>crimp butt splice into the factory lead, solder onto the factory lead</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -20241,7 +20352,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wires: 139   Connectors / ends: 59   Splices: 20   Spare cavities: 60</t>
+          <t>Wires: 140   Connectors / ends: 59   Splices: 20   Spare cavities: 60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harness ownership: one plug = one harness, 22 wires moved; pin chart devices-by-harness page; row 182 closed (Dan 2026-11-01) (#465)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-cabin-wirelist.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Y$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Connectors'!$A$1:$I$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Splices'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$61</definedName>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y140"/>
+  <dimension ref="A1:Y141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>ST185-AntiTheft</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4380,7 +4380,7 @@
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on ECU-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on ECU-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm); harness ownership (Dan 2026-11-01): was AntiTheft via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -9361,7 +9361,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>ST185-AB-engine wc_h_lam_be at DRB102-ENGINE 79, to splice SP-CANH-LAM; SP-CANH also joins ST185-CAN</t>
+          <t>ST185-AB-engine wc_h_lam_be at DRB102-ENGINE 79, to splice SP-CANH-LAM; SP-CANH also joins ST185-CAN, ST185-CSB3</t>
         </is>
       </c>
       <c r="W80" t="inlineStr"/>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>ST185-AB-engine wc_l_lam_be at DRB102-ENGINE 80, to splice SP-CANL-LAM; SP-CANL also joins ST185-CAN</t>
+          <t>ST185-AB-engine wc_l_lam_be at DRB102-ENGINE 80, to splice SP-CANL-LAM; SP-CANL also joins ST185-CAN, ST185-CSB3</t>
         </is>
       </c>
       <c r="W81" t="inlineStr"/>
@@ -11646,7 +11646,7 @@
       </c>
       <c r="T101" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U101" t="inlineStr">
@@ -11663,7 +11663,7 @@
       <c r="X101" t="inlineStr"/>
       <c r="Y101" t="inlineStr">
         <is>
-          <t>POWER box (glove box) relay R2 EFI main, pin 85 | owner proposed: longer half (drawn today as w76 on ECU-cabin, 370 mm; w76_cp on CabinPower, 400 mm)</t>
+          <t>POWER box (glove box) relay R2 EFI main, pin 85 | owner proposed: longer half (drawn today as w76 on ECU-cabin, 370 mm; w76_cp on CabinPower, 400 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -11864,7 +11864,7 @@
       </c>
       <c r="T103" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U103" t="inlineStr">
@@ -11881,7 +11881,7 @@
       <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) relay M14 ETB power, pin 85 | owner proposed: longer half (drawn today as w81 on ECU-cabin, 380 mm; w81_cp on CabinPower, 400 mm)</t>
+          <t>LOGIC box (glove box) relay M14 ETB power, pin 85 | owner proposed: longer half (drawn today as w81 on ECU-cabin, 380 mm; w81_cp on CabinPower, 400 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="T104" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U104" t="inlineStr">
@@ -11984,7 +11984,7 @@
       <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w82_ac on CabinPower, 400 mm; w82 on ECU-cabin, 340 mm)</t>
+          <t>owner proposed: longer half (drawn today as w82_ac on CabinPower, 400 mm; w82 on ECU-cabin, 340 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12391,7 +12391,7 @@
       </c>
       <c r="T108" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U108" t="inlineStr">
@@ -12408,7 +12408,7 @@
       <c r="X108" t="inlineStr"/>
       <c r="Y108" t="inlineStr">
         <is>
-          <t>CAN-Lambda +12 V | CAN-Lambda +12 V | owner proposed: longer half (drawn today as w_lam12_cp on CabinPower, 250 mm; w_lam12_bc on ECU-cabin, 120 mm)</t>
+          <t>CAN-Lambda +12 V | CAN-Lambda +12 V | owner proposed: longer half (drawn today as w_lam12_cp on CabinPower, 250 mm; w_lam12_bc on ECU-cabin, 120 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12712,7 @@
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
@@ -12733,7 +12733,7 @@
       <c r="X111" t="inlineStr"/>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse COP 10A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse COP 10A | Coil +12 V feed | owner proposed: longer half (drawn today as w_cop_pwr_ac on ECU-cabin, 180 mm; w_cop_pwr_c_ac on CabinPower, 250 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -12823,7 +12823,7 @@
       </c>
       <c r="T112" t="inlineStr">
         <is>
-          <t>ST185-CabinPower</t>
+          <t>ST185-AB-cabin</t>
         </is>
       </c>
       <c r="U112" t="inlineStr">
@@ -12844,7 +12844,7 @@
       <c r="X112" t="inlineStr"/>
       <c r="Y112" t="inlineStr">
         <is>
-          <t>LOGIC box (glove box) fuse INJ 7.5A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm)</t>
+          <t>LOGIC box (glove box) fuse INJ 7.5A | Injector +12 V feed | owner proposed: longer half (drawn today as w_inj_pwr_ac on ECU-cabin, 180 mm; w_inj_pwr_c_ac on CabinPower, 250 mm); harness ownership (Dan 2026-11-01): was CabinPower via AB-cabin</t>
         </is>
       </c>
     </row>
@@ -13683,89 +13683,85 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>cab_aps1_sh</t>
+          <t>w_strl_c</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>NC, floats</t>
+          <t>RB4</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>drain</t>
+          <t>wire</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Starter solenoid S</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Shield</t>
-        </is>
-      </c>
-      <c r="J121" t="inlineStr"/>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>(cable core)</t>
-        </is>
-      </c>
-      <c r="M121" t="inlineStr">
-        <is>
-          <t>CAB-APS1</t>
-        </is>
-      </c>
-      <c r="N121" t="inlineStr">
-        <is>
-          <t>55A1831-20-2/4/6-9</t>
-        </is>
-      </c>
-      <c r="O121" t="inlineStr"/>
+          <t>J1128-TXL-12-RED</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>crimp butt splice into the factory lead</t>
+        </is>
+      </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>solder splice SP-SHIELD-A-APS</t>
+          <t>0460-220-1231</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>cab_aps1 screen (floats at the device end)</t>
+          <t>OEM R/B No.4 starter relay pin 4 (RH kick), starter out</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>via SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13775,26 +13771,30 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS</t>
-        </is>
-      </c>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
-      <c r="X121" t="inlineStr"/>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_strl_e at DRB102-ENGINE 3, to STARTER-TRIGGER 1</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>R/B No.4 starter relay pin 4, RH kick; OEM colour B; EWD 1993 p.66; crimp butt splice into the factory lead at R/B No.4 pin 4</t>
+        </is>
+      </c>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>Screen floats at this end: cut back and seal under heat-shrink | screen floats at the far end; pedal branch length estimated from OEM body dimensions + 10 % (990 mm ECU-A</t>
+          <t>OEM starter relay output (was EB1-2). New wire to the starter S terminal. | (firewall bulkhead, RH) | Starter S crosses the firewall on its own DRB102 size-12 cavity (Dan 2026-10-27); 12 AWG: the DRB size-12 contact takes 12-14 AWG, solenoid S draw is brief, OEM lead is lighter; harness ownership (Dan 2026-11-01): was CabinPower</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>cab_aps_sh</t>
+          <t>cab_aps1_sh</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -13829,7 +13829,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>CAB-APS2</t>
+          <t>CAB-APS1</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>cab_aps2 screen (floats at the device end)</t>
+          <t>cab_aps1 screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -13905,7 +13905,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_sh_ac</t>
+          <t>cab_aps_sh</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -13940,7 +13940,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -13951,7 +13951,7 @@
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>840</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -13961,33 +13961,33 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>CAB-FSPUR-FR-AC</t>
+          <t>CAB-APS2</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>55A1811-20-9-9CS2275</t>
+          <t>55A1831-20-2/4/6-9</t>
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
-          <t>solder splice SP-SHIELD-A-WSF</t>
+          <t>solder splice SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac screen (floats at the device end)</t>
+          <t>cab_aps2 screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>via SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>via SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
@@ -13997,36 +13997,36 @@
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF</t>
+          <t>SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
       <c r="Y123" t="inlineStr">
         <is>
-          <t>Screen floats at this end: cut back and seal under heat-shrink | tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+          <t>Screen floats at this end: cut back and seal under heat-shrink | screen floats at the far end; pedal branch length estimated from OEM body dimensions + 10 % (990 mm ECU-A</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>w19</t>
+          <t>cab_fspur_fr_sh_ac</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>legs of SP-8V</t>
+          <t>NC, floats</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -14036,69 +14036,69 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>SP-8V</t>
+          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>drain</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>+8 V sensor supply</t>
+          <t>FR wheel spd shield</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>500</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-ORANGE</t>
-        </is>
-      </c>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>solder splice</t>
-        </is>
-      </c>
+          <t>(cable core)</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>CAB-FSPUR-FR-AC</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>55A1811-20-9-9CS2275</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>solder splice SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-8V: +8 V supply, cam sensor + gearbox speed sensor only (ECU A6)</t>
+          <t>cab_fspur_fr_ac screen (floats at the device end)</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>via SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>8V</t>
+          <t>WSSF</t>
         </is>
       </c>
       <c r="T124" t="inlineStr">
@@ -14108,27 +14108,31 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>SP-8V</t>
+          <t>SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>dash branch (front WS inline)</t>
         </is>
       </c>
       <c r="X124" t="inlineStr"/>
-      <c r="Y124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>Screen floats at this end: cut back and seal under heat-shrink | tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>w_a5_pin</t>
+          <t>w19</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>legs of SP-A5</t>
+          <t>legs of SP-8V</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -14143,12 +14147,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>SP-A5</t>
+          <t>SP-8V</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -14158,17 +14162,17 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
+          <t>+8 V sensor supply</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -14178,7 +14182,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-RED</t>
+          <t>J1128-TXL-20-ORANGE</t>
         </is>
       </c>
       <c r="M125" t="inlineStr"/>
@@ -14190,12 +14194,12 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
+          <t>ECU splice point - SP-8V: +8 V supply, cam sensor + gearbox speed sensor only (ECU A6)</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -14205,7 +14209,7 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -14215,7 +14219,7 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>SP-A5</t>
+          <t>SP-8V</t>
         </is>
       </c>
       <c r="V125" t="inlineStr"/>
@@ -14225,21 +14229,17 @@
         </is>
       </c>
       <c r="X125" t="inlineStr"/>
-      <c r="Y125" t="inlineStr">
-        <is>
-          <t>ECU main +12 V | ECU main +12 V</t>
-        </is>
-      </c>
+      <c r="Y125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>w_ac_psw_in</t>
+          <t>w_a5_pin</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>legs of SP-AC-PSW</t>
+          <t>legs of SP-A5</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -14249,17 +14249,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-A5</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -14269,27 +14269,27 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="M126" t="inlineStr"/>
@@ -14301,22 +14301,22 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the switch's </t>
+          <t>3-1447221-3</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>At A/C amp - SP-AC-PSW: A/C pressure switch output</t>
+          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>OEM A5, factory Y-R lead</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SW12</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14326,35 +14326,31 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>SP-AC-PSW</t>
+          <t>SP-A5</t>
         </is>
       </c>
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="X126" t="inlineStr">
-        <is>
-          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo); OEM colour Y-R (factory wiring; new wire here); EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R); new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
-        </is>
-      </c>
+          <t>at ECU-A plug</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr"/>
       <c r="Y126" t="inlineStr">
         <is>
-          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152. | owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on ECU-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
+          <t>ECU main +12 V | ECU main +12 V</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>w_amb_rtn</t>
+          <t>w_ac_psw_in</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>legs of SP-AC-SG</t>
+          <t>legs of SP-AC-PSW</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -14364,17 +14360,17 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -14384,7 +14380,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Gnd</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -14399,12 +14395,12 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-YELLOW</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="M127" t="inlineStr"/>
@@ -14416,22 +14412,22 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
+          <t xml:space="preserve">new-wire run terminated at the switch's </t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>SP-AC-SG - cabin A/C sensor common (replaces E10; A32-15, A24-3, A21, A18-2 stay factory)</t>
+          <t>At A/C amp - SP-AC-PSW: A/C pressure switch output</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
+          <t>OEM A5, factory Y-R lead</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>AMB</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14441,31 +14437,35 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>SP-AC-SG</t>
+          <t>SP-AC-PSW</t>
         </is>
       </c>
       <c r="V127" t="inlineStr"/>
-      <c r="W127" t="inlineStr"/>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo); OEM colour Y-R (factory wiring; new wire here); EWD 1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R); new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
         <is>
-          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152. | owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on ECU-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>w_trig2_pin</t>
+          <t>w_amb_rtn</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>legs of SP-CAM</t>
+          <t>legs of SP-AC-SG</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -14475,17 +14475,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>SP-CAM</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -14495,12 +14495,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Cam sensor signal</t>
+          <t>Gnd</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -14510,12 +14510,12 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-YELLOW</t>
         </is>
       </c>
       <c r="M128" t="inlineStr"/>
@@ -14527,22 +14527,22 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t xml:space="preserve">new-wire run terminated at the sensor's </t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>At the ECU plugs - SP-CAM: cam signal + 1.8k pull-up to +8V</t>
+          <t>SP-AC-SG - cabin A/C sensor common (replaces E10; A32-15, A24-3, A21, A18-2 stay factory)</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>OEM ambient air temp sensor A1 pin 1 (front, 6 in pigtail)</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>AMB</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
@@ -14552,27 +14552,31 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>SP-CAM</t>
+          <t>SP-AC-SG</t>
         </is>
       </c>
       <c r="V128" t="inlineStr"/>
-      <c r="W128" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
-      <c r="X128" t="inlineStr"/>
-      <c r="Y128" t="inlineStr"/>
+      <c r="W128" t="inlineStr"/>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>Ambient air temp sensor A1 pin 1 (6 in pigtail, B9); OEM colour Y; EWD 1993 p.211; new-wire run terminated at the sensor's own mating plug; 6 in OEM pigtail stays</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>Row 164: E10 sensor-common dies under B9. Cabin splice SP-AC-SG kept. Factory Y-R is the A/C pressure-switch output (A5-4 through joiner E10 to A18-13), not sensor ground; sensor common is Y (1990 ST185 EWD p.150 / p.152).</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>w_csbg_ac</t>
+          <t>w_trig2_pin</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>legs of SP-CSB-GND</t>
+          <t>legs of SP-CAM</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -14582,17 +14586,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>SP-CSB-GND</t>
+          <t>SP-CAM</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -14602,12 +14606,12 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Gnd to CSB3, opto board</t>
+          <t>Cam sensor signal</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14617,12 +14621,12 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-BLACK</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M129" t="inlineStr"/>
@@ -14634,22 +14638,22 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>CSB3 ground splice - CSB3 pin 2, opto board COM and stalk ground</t>
+          <t>At the ECU plugs - SP-CAM: cam signal + 1.8k pull-up to +8V</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14659,35 +14663,27 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>SP-CSB-GND</t>
-        </is>
-      </c>
-      <c r="V129" t="inlineStr">
-        <is>
-          <t>SP-CSB-GND also joins ST185-CSB3</t>
-        </is>
-      </c>
+          <t>SP-CAM</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr">
         <is>
-          <t>glove-box POWER box to the CSB3 branch</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X129" t="inlineStr"/>
-      <c r="Y129" t="inlineStr">
-        <is>
-          <t>M8 ring lug on the POWER box battery-negative bar (R213: CSB3, opto board and cruise ladder never on chassis or the ECU ground) | (CSB3 loom, under centre cluster) | est length; runs with the CSB3 +12 V (w_csb12, LOGIC CSB 5A) (R217)</t>
-        </is>
-      </c>
+      <c r="Y129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>w_fl_sig_pin</t>
+          <t>w_csbg_ac</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>legs of SP-FUEL-LVL</t>
+          <t>legs of SP-CSB-GND</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -14697,17 +14693,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL</t>
+          <t>SP-CSB-GND</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -14717,12 +14713,12 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Fuel level signal</t>
+          <t>Gnd to CSB3, opto board</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14732,12 +14728,12 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-20-BLACK</t>
         </is>
       </c>
       <c r="M130" t="inlineStr"/>
@@ -14749,22 +14745,22 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL - fuel sender signal + 470R pull-up to ECU-B B24</t>
+          <t>CSB3 ground splice - CSB3 pin 2, opto board COM and stalk ground</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>FLVL</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14774,23 +14770,35 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>SP-FUEL-LVL</t>
-        </is>
-      </c>
-      <c r="V130" t="inlineStr"/>
-      <c r="W130" t="inlineStr"/>
+          <t>SP-CSB-GND</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>SP-CSB-GND also joins ST185-CSB3</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>glove-box POWER box to the CSB3 branch</t>
+        </is>
+      </c>
       <c r="X130" t="inlineStr"/>
-      <c r="Y130" t="inlineStr"/>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>M8 ring lug on the POWER box battery-negative bar (R213: CSB3, opto board and cruise ladder never on chassis or the ECU ground) | (CSB3 loom, under centre cluster) | est length; runs with the CSB3 +12 V (w_csb12, LOGIC CSB 5A) (R217)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>w66</t>
+          <t>w_fl_sig_pin</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>legs of SP-GND-ECU</t>
+          <t>legs of SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -14800,17 +14808,17 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>POWER-NEG-BAR</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>24</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>SP-GND-ECU</t>
+          <t>SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -14820,27 +14828,27 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>ECU power ground</t>
+          <t>Fuel level signal</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>White</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>310</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>J1128-TXL-10-BLACK</t>
+          <t>J1128-TXL-20-WHITE</t>
         </is>
       </c>
       <c r="M131" t="inlineStr"/>
@@ -14852,22 +14860,22 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-GND-ECU: ECU power ground (A25 A34 B25 B34) to the NEG bar</t>
+          <t>SP-FUEL-LVL - fuel sender signal + 470R pull-up to ECU-B B24</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>POWER box NEG bar M8 stud (glove box)</t>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>GND</t>
+          <t>FLVL</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14877,31 +14885,23 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>SP-GND-ECU</t>
+          <t>SP-FUEL-LVL</t>
         </is>
       </c>
       <c r="V131" t="inlineStr"/>
-      <c r="W131" t="inlineStr">
-        <is>
-          <t>ECU to the glove-box POWER box</t>
-        </is>
-      </c>
+      <c r="W131" t="inlineStr"/>
       <c r="X131" t="inlineStr"/>
-      <c r="Y131" t="inlineStr">
-        <is>
-          <t>M8 ring lug on the POWER box battery-negative bar (R216): the ECU grounds only, nothing else | est length; the ONE ECU ground return (DECISIONS R216)</t>
-        </is>
-      </c>
+      <c r="Y131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>w_rev_sw_c</t>
+          <t>w66</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>legs of SP-REV</t>
+          <t>legs of SP-GND-ECU</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -14911,17 +14911,17 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>DRB102-CABIN</t>
+          <t>POWER-NEG-BAR</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>Lug</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>SP-REV</t>
+          <t>SP-GND-ECU</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -14931,27 +14931,27 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Switched +12 V from reverse switch</t>
+          <t>ECU power ground</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>570</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>J1128-TXL-16-YELLOW</t>
+          <t>J1128-TXL-10-BLACK</t>
         </is>
       </c>
       <c r="M132" t="inlineStr"/>
@@ -14963,22 +14963,22 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>0460-202-1631</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
+          <t>ECU splice point - SP-GND-ECU: ECU power ground (A25 A34 B25 B34) to the NEG bar</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>DRB102 receptacle (RH firewall)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14988,31 +14988,31 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>SP-REV</t>
-        </is>
-      </c>
-      <c r="V132" t="inlineStr">
-        <is>
-          <t>ST185-AB-engine w_sw7_e at DRB102-ENGINE 78, to REV-SW 1</t>
-        </is>
-      </c>
-      <c r="W132" t="inlineStr"/>
+          <t>SP-GND-ECU</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr"/>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>ECU to the glove-box POWER box</t>
+        </is>
+      </c>
       <c r="X132" t="inlineStr"/>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>Circuit 11: switch out tapped to opto IN2; lamps stay on the factory IG2-13 run.</t>
+          <t>M8 ring lug on the POWER box battery-negative bar (R216): the ECU grounds only, nothing else | est length; the ONE ECU ground return (DECISIONS R216)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>w_drain_ecu_a</t>
+          <t>w_rev_sw_c</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A</t>
+          <t>legs of SP-REV</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -15022,17 +15022,17 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>ECU-A</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>78</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A</t>
+          <t>SP-REV</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -15042,27 +15042,27 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Shield drain</t>
+          <t>Switched +12 V from reverse switch</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J1128-TXL-16-YELLOW</t>
         </is>
       </c>
       <c r="M133" t="inlineStr"/>
@@ -15074,22 +15074,22 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>0460-202-1631</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
+          <t>SP-REV - reverse switch signal to CSB3 opto IN2 and IG2-13 lamps</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>Link G4X plug A (centre dash)</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>SHLD</t>
+          <t>REV</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -15099,31 +15099,31 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A</t>
-        </is>
-      </c>
-      <c r="V133" t="inlineStr"/>
-      <c r="W133" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
+          <t>SP-REV</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_sw7_e at DRB102-ENGINE 78, to REV-SW 1</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr"/>
       <c r="X133" t="inlineStr"/>
       <c r="Y133" t="inlineStr">
         <is>
-          <t>build (R30): the crank drain is the one crimped into A7; the other drains are soldered onto it 6 mm behind the plug</t>
+          <t>Circuit 11: switch out tapped to opto IN2; lamps stay on the factory IG2-13 run.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>w_shd_a_aps</t>
+          <t>w_drain_ecu_a</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A-APS</t>
+          <t>legs of SP-SHIELD-A</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -15133,22 +15133,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A</t>
+          <t>ECU-A</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -15168,7 +15168,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -15185,17 +15185,17 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>solder splice</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
+          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
+          <t>Link G4X plug A (centre dash)</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
@@ -15210,27 +15210,31 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-APS / SP-SHIELD-A</t>
+          <t>SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V134" t="inlineStr"/>
-      <c r="W134" t="inlineStr"/>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>at ECU-A plug</t>
+        </is>
+      </c>
       <c r="X134" t="inlineStr"/>
       <c r="Y134" t="inlineStr">
         <is>
-          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+          <t>build (R30): the crank drain is the one crimped into A7; the other drains are soldered onto it 6 mm behind the plug</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>w_shd_a_wsf</t>
+          <t>w_shd_a_aps</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-A-WSF</t>
+          <t>legs of SP-SHIELD-A-APS</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -15250,7 +15254,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -15275,7 +15279,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>450</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -15297,7 +15301,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
+          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -15317,7 +15321,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>SP-SHIELD-A-WSF / SP-SHIELD-A</t>
+          <t>SP-SHIELD-A-APS / SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V135" t="inlineStr"/>
@@ -15332,12 +15336,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>w_drain_ecu_b</t>
+          <t>w_shd_a_wsf</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B</t>
+          <t>legs of SP-SHIELD-A-WSF</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -15347,27 +15351,27 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>legs of SP-SHIELD-A</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B</t>
+          <t>SP-SHIELD-A-WSF &gt; SP-SHIELD-A</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>link</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Shield drain B</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -15382,7 +15386,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -15399,17 +15403,17 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
+          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>6 mm behind the ECU-A plug - SP-SHIELD-A: drains to A7</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
@@ -15424,23 +15428,27 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B</t>
+          <t>SP-SHIELD-A-WSF / SP-SHIELD-A</t>
         </is>
       </c>
       <c r="V136" t="inlineStr"/>
       <c r="W136" t="inlineStr"/>
       <c r="X136" t="inlineStr"/>
-      <c r="Y136" t="inlineStr"/>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>w_shd_b_wsr</t>
+          <t>w_drain_ecu_b</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B-WSR</t>
+          <t>legs of SP-SHIELD-B</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -15450,22 +15458,22 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>legs of SP-SHIELD-B</t>
+          <t>ECU-B</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B-WSR &gt; SP-SHIELD-B</t>
+          <t>SP-SHIELD-B</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>trunk</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -15485,7 +15493,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -15502,17 +15510,17 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>solder splice</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>At the rear WS inline - SP-SHIELD-B-WSR: rear wheel-speed drains</t>
+          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
@@ -15527,27 +15535,23 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>SP-SHIELD-B-WSR / SP-SHIELD-B</t>
+          <t>SP-SHIELD-B</t>
         </is>
       </c>
       <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr"/>
-      <c r="Y137" t="inlineStr">
-        <is>
-          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
-        </is>
-      </c>
+      <c r="Y137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>w78</t>
+          <t>w_shd_b_wsr</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>legs of SP-SW12</t>
+          <t>legs of SP-SHIELD-B-WSR</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -15557,7 +15561,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>legs of SP-A5</t>
+          <t>legs of SP-SHIELD-B</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -15567,7 +15571,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>SP-SW12 &gt; SP-A5</t>
+          <t>SP-SHIELD-B-WSR &gt; SP-SHIELD-B</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -15577,27 +15581,27 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
+          <t>Shield drain B</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>230</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>J1128-TXL-18-RED</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
@@ -15614,17 +15618,17 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-SW12: switched +12 V (LOGIC SW12)</t>
+          <t>At the rear WS inline - SP-SHIELD-B-WSR: rear wheel-speed drains</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
+          <t>6 mm behind the ECU-B plug - SP-SHIELD-B: drains to B17</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15634,26 +15638,22 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>SP-SW12 / SP-A5</t>
+          <t>SP-SHIELD-B-WSR / SP-SHIELD-B</t>
         </is>
       </c>
       <c r="V138" t="inlineStr"/>
-      <c r="W138" t="inlineStr">
-        <is>
-          <t>at ECU-A plug</t>
-        </is>
-      </c>
+      <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr"/>
       <c r="Y138" t="inlineStr">
         <is>
-          <t>ECU main +12 V | ECU main +12 V</t>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>w_rail_sp_sw12_c</t>
+          <t>w78</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -15668,27 +15668,27 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>DRB102-CABIN</t>
+          <t>legs of SP-A5</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>SP-SW12</t>
+          <t>SP-SW12 &gt; SP-A5</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>trunk</t>
+          <t>link</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse (+ IG2 wake diode)</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -15703,7 +15703,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>0460-202-1631</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>DRB102 receptacle (RH firewall)</t>
+          <t>ECU splice point - SP-A5: ECU main feed (SW12 + IG2 diode)</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
@@ -15745,35 +15745,31 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>SP-SW12</t>
-        </is>
-      </c>
-      <c r="V139" t="inlineStr">
-        <is>
-          <t>ST185-AB-engine w_rail_sp_sw12_e at DRB102-ENGINE 30, to splice SP-SW12-ENG</t>
-        </is>
-      </c>
+          <t>SP-SW12 / SP-A5</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr">
         <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="X139" t="inlineStr"/>
       <c r="Y139" t="inlineStr">
         <is>
-          <t>+12 V boost + flex | +12 V boost + flex</t>
+          <t>ECU main +12 V | ECU main +12 V</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>w_tach</t>
+          <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>legs of SP-TACH</t>
+          <t>legs of SP-SW12</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -15783,17 +15779,17 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ECU-B</t>
+          <t>DRB102-CABIN</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
+          <t>SP-SW12</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -15803,27 +15799,27 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Engine speed (tacho)</t>
+          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>520</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>J1128-TXL-20-WHITE</t>
+          <t>J1128-TXL-18-RED</t>
         </is>
       </c>
       <c r="M140" t="inlineStr"/>
@@ -15835,22 +15831,22 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>0460-202-1631</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>SP-TACH - Ign 8 tacho to A15 pin 18 and 4.7k lock-sensor tap</t>
+          <t>ECU splice point - SP-SW12: switched +12 V (LOGIC SW12)</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
+          <t>DRB102 receptacle (RH firewall)</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>TACH</t>
+          <t>SW12</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15860,24 +15856,139 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>SP-TACH</t>
-        </is>
-      </c>
-      <c r="V140" t="inlineStr"/>
+          <t>SP-SW12</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>ST185-AB-engine w_rail_sp_sw12_e at DRB102-ENGINE 30, to splice SP-SW12-ENG</t>
+        </is>
+      </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
       <c r="Y140" t="inlineStr">
         <is>
+          <t>+12 V boost + flex | +12 V boost + flex</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>w_tach</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>legs of SP-TACH</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>ECU-B</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>SP-TACH</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>trunk</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Engine speed (tacho)</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>J1128-TXL-20-WHITE</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>solder splice</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>3-1447221-4</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>SP-TACH - Ign 8 tacho to A15 pin 18 and 4.7k lock-sensor tap</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>TACH</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>SP-TACH</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr"/>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr">
+        <is>
           <t>Ign 8 (ECU-B 10) tacho. Split at SP-TACH: pin 18 plus 4.7k to pin 9 (OPEN-ITEMS History 2026-10-21 N61).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y140"/>
+  <autoFilter ref="A1:Y141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16278,7 +16389,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H9" t="n">
         <v>37</v>
@@ -17144,11 +17255,11 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>solder onto the factory lead</t>
+          <t>crimp butt splice into the factory lead, solder onto the factory lead</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -20241,7 +20352,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wires: 139   Connectors / ends: 59   Splices: 20   Spare cavities: 60</t>
+          <t>Wires: 140   Connectors / ends: 59   Splices: 20   Spare cavities: 60</t>
         </is>
       </c>
     </row>

</xml_diff>